<commit_message>
新品 iPhone 18 Pro/AirPods 5/Watch S12/Ultra 4 納入統計，第 6/16 頁改日報新格式（版本號 1.6.0）
- C6_AIRPODS 加 AirPods 5（6348），第 1 頁新增 5 個新機種列
- 第 6/16 頁列項改為日報格式：零售/訂單出貨/訂金營業額、ACPP、各機種保固加總搭售率、AirPods
- Apple/3PP/ACPP 毛利改為重現 ERP BI「02/03-日報 毛利額 含稅」

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/週報模板.xlsx
+++ b/週報模板.xlsx
@@ -750,7 +750,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="185">
+  <cellXfs count="186">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1291,6 +1291,9 @@
     </xf>
     <xf numFmtId="0" fontId="31" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5552,7 +5555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="27" bestFit="1" customWidth="1" style="106" min="1" max="1"/>
@@ -5579,586 +5582,475 @@
       </c>
       <c r="E1" s="108" t="n"/>
     </row>
-    <row r="2">
+    <row r="2" s="106">
       <c r="A2" s="76" t="inlineStr">
         <is>
-          <t>總營業額</t>
-        </is>
-      </c>
-      <c r="B2" s="77" t="n">
-        <v>37865386</v>
-      </c>
-      <c r="C2" s="77" t="n">
-        <v>44763710</v>
-      </c>
-      <c r="D2" s="77" t="n">
-        <v>6898324</v>
-      </c>
-      <c r="E2" s="78" t="n">
-        <v>0.182</v>
-      </c>
-    </row>
-    <row r="3">
+          <t>總營業額(a + c + d + e)</t>
+        </is>
+      </c>
+      <c r="B2" s="77" t="n"/>
+      <c r="C2" s="77" t="n"/>
+      <c r="D2" s="77" t="n"/>
+      <c r="E2" s="78" t="n"/>
+    </row>
+    <row r="3" s="106">
       <c r="A3" s="76" t="inlineStr">
         <is>
-          <t>零售營業額</t>
-        </is>
-      </c>
-      <c r="B3" s="77" t="n">
-        <v>37865386</v>
-      </c>
-      <c r="C3" s="77" t="n">
-        <v>44763710</v>
-      </c>
-      <c r="D3" s="77" t="n">
-        <v>6898324</v>
-      </c>
-      <c r="E3" s="78" t="n">
-        <v>0.182</v>
-      </c>
-    </row>
-    <row r="4">
+          <t>零售營業額(a)</t>
+        </is>
+      </c>
+      <c r="B3" s="77" t="n"/>
+      <c r="C3" s="77" t="n"/>
+      <c r="D3" s="77" t="n"/>
+      <c r="E3" s="78" t="n"/>
+    </row>
+    <row r="4" s="106">
       <c r="A4" s="76" t="inlineStr">
         <is>
-          <t>專案營業額</t>
-        </is>
-      </c>
-      <c r="B4" s="0" t="n"/>
-      <c r="C4" s="0" t="n"/>
-      <c r="D4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="79" t="n"/>
-    </row>
-    <row r="5">
+          <t>訂單出貨金額(b)</t>
+        </is>
+      </c>
+      <c r="B4" s="77" t="n"/>
+      <c r="C4" s="77" t="n"/>
+      <c r="D4" s="77" t="n"/>
+      <c r="E4" s="78" t="n"/>
+    </row>
+    <row r="5" s="106">
       <c r="A5" s="76" t="inlineStr">
         <is>
+          <t>當日零售營業收入(a + b)</t>
+        </is>
+      </c>
+      <c r="B5" s="77" t="n"/>
+      <c r="C5" s="77" t="n"/>
+      <c r="D5" s="77" t="n"/>
+      <c r="E5" s="78" t="n"/>
+    </row>
+    <row r="6" s="106">
+      <c r="A6" s="76" t="inlineStr">
+        <is>
+          <t>零售訂金營業額(c)</t>
+        </is>
+      </c>
+      <c r="B6" s="77" t="n"/>
+      <c r="C6" s="77" t="n"/>
+      <c r="D6" s="77" t="n"/>
+      <c r="E6" s="78" t="n"/>
+    </row>
+    <row r="7" s="106">
+      <c r="A7" s="76" t="inlineStr">
+        <is>
+          <t>專案營業額(d)</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n"/>
+      <c r="C7" s="0" t="n"/>
+      <c r="D7" s="0" t="n"/>
+      <c r="E7" s="79" t="n"/>
+    </row>
+    <row r="8" s="106">
+      <c r="A8" s="76" t="inlineStr">
+        <is>
           <t>Apple 主機營業額</t>
         </is>
       </c>
-      <c r="B5" s="77" t="n">
-        <v>28454402</v>
-      </c>
-      <c r="C5" s="77" t="n">
-        <v>35187994</v>
-      </c>
-      <c r="D5" s="77" t="n">
-        <v>6733592</v>
-      </c>
-      <c r="E5" s="80" t="n">
-        <v>0.24</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="76" t="inlineStr">
+      <c r="B8" s="77" t="n"/>
+      <c r="C8" s="77" t="n"/>
+      <c r="D8" s="77" t="n"/>
+      <c r="E8" s="80" t="n"/>
+    </row>
+    <row r="9" s="106">
+      <c r="A9" s="76" t="inlineStr">
         <is>
           <t>Apple 配件營業額</t>
         </is>
       </c>
-      <c r="B6" s="77" t="n">
-        <v>4953169</v>
-      </c>
-      <c r="C6" s="77" t="n">
-        <v>4304081</v>
-      </c>
-      <c r="D6" s="77" t="n">
-        <v>-649088</v>
-      </c>
-      <c r="E6" s="80" t="n">
-        <v>-0.13</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="76" t="inlineStr">
+      <c r="B9" s="77" t="n"/>
+      <c r="C9" s="77" t="n"/>
+      <c r="D9" s="77" t="n"/>
+      <c r="E9" s="80" t="n"/>
+    </row>
+    <row r="10" s="106">
+      <c r="A10" s="76" t="inlineStr">
         <is>
           <t>3PP配件營業額</t>
         </is>
       </c>
-      <c r="B7" s="77" t="n">
-        <v>3025452</v>
-      </c>
-      <c r="C7" s="77" t="n">
-        <v>4428930</v>
-      </c>
-      <c r="D7" s="77" t="n">
-        <v>1403478</v>
-      </c>
-      <c r="E7" s="78" t="n">
-        <v>0.464</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="81" t="inlineStr">
+      <c r="B10" s="77" t="n"/>
+      <c r="C10" s="77" t="n"/>
+      <c r="D10" s="77" t="n"/>
+      <c r="E10" s="78" t="n"/>
+    </row>
+    <row r="11" s="106">
+      <c r="A11" s="81" t="inlineStr">
         <is>
           <t>3PP搭售率</t>
         </is>
       </c>
-      <c r="B8" s="82" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="C8" s="82" t="n">
-        <v>0.099</v>
-      </c>
-      <c r="D8" s="82" t="n">
-        <v>0.019</v>
-      </c>
-      <c r="E8" s="83" t="n">
-        <v>0.24</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="76" t="inlineStr">
-        <is>
-          <t>SA Care 營業額</t>
-        </is>
-      </c>
-      <c r="B9" s="77" t="n">
-        <v>1806179</v>
-      </c>
-      <c r="C9" s="77" t="n">
-        <v>1814090</v>
-      </c>
-      <c r="D9" s="77" t="n">
-        <v>7911</v>
-      </c>
-      <c r="E9" s="80" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="81" t="inlineStr">
+      <c r="B11" s="82" t="n"/>
+      <c r="C11" s="82" t="n"/>
+      <c r="D11" s="82" t="n"/>
+      <c r="E11" s="83" t="n"/>
+    </row>
+    <row r="12" s="106">
+      <c r="A12" s="76" t="inlineStr">
+        <is>
+          <t>ACPP 營業額</t>
+        </is>
+      </c>
+      <c r="B12" s="77" t="n"/>
+      <c r="C12" s="77" t="n"/>
+      <c r="D12" s="77" t="n"/>
+      <c r="E12" s="80" t="n"/>
+    </row>
+    <row r="13" s="106">
+      <c r="A13" s="81" t="inlineStr">
+        <is>
+          <t>ACPP 搭售率</t>
+        </is>
+      </c>
+      <c r="B13" s="82" t="n"/>
+      <c r="C13" s="82" t="n"/>
+      <c r="D13" s="82" t="n"/>
+      <c r="E13" s="83" t="n"/>
+    </row>
+    <row r="14" s="106">
+      <c r="A14" s="76" t="inlineStr">
+        <is>
+          <t>SA Care 營業額(e)</t>
+        </is>
+      </c>
+      <c r="B14" s="77" t="n"/>
+      <c r="C14" s="77" t="n"/>
+      <c r="D14" s="77" t="n"/>
+      <c r="E14" s="80" t="n"/>
+    </row>
+    <row r="15" s="106">
+      <c r="A15" s="81" t="inlineStr">
         <is>
           <t>SA Care 搭售率</t>
         </is>
       </c>
-      <c r="B10" s="82" t="n">
-        <v>0.048</v>
-      </c>
-      <c r="C10" s="82" t="n">
-        <v>0.041</v>
-      </c>
-      <c r="D10" s="82" t="n">
-        <v>-0.0072</v>
-      </c>
-      <c r="E10" s="83" t="n">
-        <v>-0.15</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="76" t="inlineStr">
+      <c r="B15" s="82" t="n"/>
+      <c r="C15" s="82" t="n"/>
+      <c r="D15" s="82" t="n"/>
+      <c r="E15" s="83" t="n"/>
+    </row>
+    <row r="16" s="106">
+      <c r="A16" s="76" t="inlineStr">
         <is>
           <t>總毛利額</t>
         </is>
       </c>
-      <c r="B11" s="77" t="n">
-        <v>4774129</v>
-      </c>
-      <c r="C11" s="77" t="n">
-        <v>6155554</v>
-      </c>
-      <c r="D11" s="77" t="n">
-        <v>1381425</v>
-      </c>
-      <c r="E11" s="80" t="n">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="76" t="inlineStr">
+      <c r="B16" s="77" t="n"/>
+      <c r="C16" s="77" t="n"/>
+      <c r="D16" s="77" t="n"/>
+      <c r="E16" s="80" t="n"/>
+    </row>
+    <row r="17" s="106">
+      <c r="A17" s="76" t="inlineStr">
         <is>
           <t>Apple 毛利額</t>
         </is>
       </c>
-      <c r="B12" s="77" t="n">
-        <v>2732116</v>
-      </c>
-      <c r="C12" s="77" t="n">
-        <v>3119165</v>
-      </c>
-      <c r="D12" s="77" t="n">
-        <v>387049</v>
-      </c>
-      <c r="E12" s="80" t="n">
-        <v>0.14</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="76" t="inlineStr">
+      <c r="B17" s="77" t="n"/>
+      <c r="C17" s="77" t="n"/>
+      <c r="D17" s="77" t="n"/>
+      <c r="E17" s="80" t="n"/>
+    </row>
+    <row r="18" s="106">
+      <c r="A18" s="76" t="inlineStr">
         <is>
           <t>3PP 毛利額</t>
         </is>
       </c>
-      <c r="B13" s="77" t="n">
-        <v>1138923</v>
-      </c>
-      <c r="C13" s="77" t="n">
-        <v>2129344</v>
-      </c>
-      <c r="D13" s="77" t="n">
-        <v>990421</v>
-      </c>
-      <c r="E13" s="80" t="n">
-        <v>0.87</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="84" t="inlineStr">
+      <c r="B18" s="77" t="n"/>
+      <c r="C18" s="77" t="n"/>
+      <c r="D18" s="77" t="n"/>
+      <c r="E18" s="80" t="n"/>
+    </row>
+    <row r="19" s="106">
+      <c r="A19" s="84" t="inlineStr">
+        <is>
+          <t>ACPP毛利額</t>
+        </is>
+      </c>
+      <c r="B19" s="74" t="n"/>
+      <c r="C19" s="74" t="n"/>
+      <c r="D19" s="74" t="n"/>
+      <c r="E19" s="85" t="n"/>
+    </row>
+    <row r="20" s="106">
+      <c r="A20" s="84" t="inlineStr">
         <is>
           <t>SA Care 毛利額</t>
         </is>
       </c>
-      <c r="B14" s="74" t="n">
-        <v>903090</v>
-      </c>
-      <c r="C14" s="74" t="n">
-        <v>907045</v>
-      </c>
-      <c r="D14" s="74" t="n">
-        <v>3955</v>
-      </c>
-      <c r="E14" s="85" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="76" t="inlineStr">
-        <is>
-          <t>CPU 台數（不含Mac mini）</t>
-        </is>
-      </c>
-      <c r="B15" s="0" t="n">
-        <v>76</v>
-      </c>
-      <c r="C15" s="0" t="n">
-        <v>72</v>
-      </c>
-      <c r="D15" s="0" t="n">
-        <v>-4</v>
-      </c>
-      <c r="E15" s="80" t="n">
-        <v>-0.05</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="76" t="inlineStr">
-        <is>
-          <t>Mac mini 台數</t>
-        </is>
-      </c>
-      <c r="B16" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="C16" s="0" t="n">
-        <v>14</v>
-      </c>
-      <c r="D16" s="0" t="n">
-        <v>-1</v>
-      </c>
-      <c r="E16" s="80" t="n">
-        <v>-0.07000000000000001</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="76" t="inlineStr">
-        <is>
-          <t>CPU 總台數</t>
-        </is>
-      </c>
-      <c r="B17" s="0" t="n">
-        <v>91</v>
-      </c>
-      <c r="C17" s="0" t="n">
-        <v>86</v>
-      </c>
-      <c r="D17" s="0" t="n">
-        <v>-5</v>
-      </c>
-      <c r="E17" s="80" t="n">
-        <v>-0.05</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="76" t="inlineStr">
+      <c r="B20" s="74" t="n"/>
+      <c r="C20" s="74" t="n"/>
+      <c r="D20" s="74" t="n"/>
+      <c r="E20" s="85" t="n"/>
+    </row>
+    <row r="21" s="106">
+      <c r="A21" s="76" t="inlineStr">
+        <is>
+          <t>CPU 台數</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n"/>
+      <c r="C21" s="0" t="n"/>
+      <c r="D21" s="0" t="n"/>
+      <c r="E21" s="80" t="n"/>
+    </row>
+    <row r="22" s="106">
+      <c r="A22" s="76" t="inlineStr">
         <is>
           <t>ACPP-MAC 套數</t>
         </is>
       </c>
-      <c r="B18" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="C18" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="D18" s="0" t="n">
-        <v>-3</v>
-      </c>
-      <c r="E18" s="80" t="n">
-        <v>-0.38</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="81" t="inlineStr">
-        <is>
-          <t>ACPP-MAC 搭售率</t>
-        </is>
-      </c>
-      <c r="B19" s="82" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="C19" s="82" t="n">
-        <v>0.058</v>
-      </c>
-      <c r="D19" s="82" t="n">
-        <v>-0.032</v>
-      </c>
-      <c r="E19" s="86" t="n">
-        <v>-0.3556</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="76" t="inlineStr">
+      <c r="B22" s="0" t="n"/>
+      <c r="C22" s="0" t="n"/>
+      <c r="D22" s="0" t="n"/>
+      <c r="E22" s="80" t="n"/>
+    </row>
+    <row r="23" s="106">
+      <c r="A23" s="76" t="inlineStr">
         <is>
           <t>SA Care for CPU 套數</t>
         </is>
       </c>
-      <c r="B20" s="0" t="n">
-        <v>42</v>
-      </c>
-      <c r="C20" s="0" t="n">
-        <v>32</v>
-      </c>
-      <c r="D20" s="0" t="n">
-        <v>-10</v>
-      </c>
-      <c r="E20" s="80" t="n">
-        <v>-0.24</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="81" t="inlineStr">
-        <is>
-          <t>SA Care for CPU 搭售率</t>
-        </is>
-      </c>
-      <c r="B21" s="82" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="C21" s="82" t="n">
-        <v>0.372</v>
-      </c>
-      <c r="D21" s="82" t="n">
-        <v>-0.08799999999999999</v>
-      </c>
-      <c r="E21" s="86" t="n">
-        <v>-0.1913</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="76" t="inlineStr">
+      <c r="B23" s="0" t="n"/>
+      <c r="C23" s="0" t="n"/>
+      <c r="D23" s="0" t="n"/>
+      <c r="E23" s="80" t="n"/>
+    </row>
+    <row r="24" s="106">
+      <c r="A24" s="81" t="inlineStr">
+        <is>
+          <t>保固加總 CPU 搭售率</t>
+        </is>
+      </c>
+      <c r="B24" s="87" t="n"/>
+      <c r="C24" s="87" t="n"/>
+      <c r="D24" s="87" t="n"/>
+      <c r="E24" s="86" t="n"/>
+    </row>
+    <row r="25" s="106">
+      <c r="A25" s="76" t="inlineStr">
         <is>
           <t>iPad 台數</t>
         </is>
       </c>
-      <c r="B22" s="0" t="n">
-        <v>232</v>
-      </c>
-      <c r="C22" s="0" t="n">
-        <v>250</v>
-      </c>
-      <c r="D22" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="E22" s="80" t="n">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="76" t="inlineStr">
+      <c r="B25" s="0" t="n"/>
+      <c r="C25" s="0" t="n"/>
+      <c r="D25" s="0" t="n"/>
+      <c r="E25" s="80" t="n"/>
+    </row>
+    <row r="26" s="106">
+      <c r="A26" s="76" t="inlineStr">
+        <is>
+          <t>ACPP-iPad 套數</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n"/>
+      <c r="C26" s="0" t="n"/>
+      <c r="D26" s="0" t="n"/>
+      <c r="E26" s="80" t="n"/>
+    </row>
+    <row r="27" s="106">
+      <c r="A27" s="76" t="inlineStr">
         <is>
           <t>SA Care for iPad 套數</t>
         </is>
       </c>
-      <c r="B23" s="0" t="n">
-        <v>120</v>
-      </c>
-      <c r="C23" s="0" t="n">
-        <v>132</v>
-      </c>
-      <c r="D23" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="E23" s="80" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="81" t="inlineStr">
-        <is>
-          <t>SA Care for iPad 搭售率</t>
-        </is>
-      </c>
-      <c r="B24" s="82" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="C24" s="82" t="n">
-        <v>0.528</v>
-      </c>
-      <c r="D24" s="87" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E24" s="83" t="n">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="76" t="inlineStr">
+      <c r="B27" s="0" t="n"/>
+      <c r="C27" s="0" t="n"/>
+      <c r="D27" s="0" t="n"/>
+      <c r="E27" s="80" t="n"/>
+    </row>
+    <row r="28" s="106">
+      <c r="A28" s="81" t="inlineStr">
+        <is>
+          <t>保固加總 iPad 搭售率</t>
+        </is>
+      </c>
+      <c r="B28" s="87" t="n"/>
+      <c r="C28" s="87" t="n"/>
+      <c r="D28" s="87" t="n"/>
+      <c r="E28" s="83" t="n"/>
+    </row>
+    <row r="29" s="106">
+      <c r="A29" s="76" t="inlineStr">
         <is>
           <t>iPhone 台數</t>
         </is>
       </c>
-      <c r="B25" s="0" t="n">
-        <v>452</v>
-      </c>
-      <c r="C25" s="0" t="n">
-        <v>646</v>
-      </c>
-      <c r="D25" s="0" t="n">
-        <v>194</v>
-      </c>
-      <c r="E25" s="80" t="n">
-        <v>0.43</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="76" t="inlineStr">
+      <c r="B29" s="0" t="n"/>
+      <c r="C29" s="0" t="n"/>
+      <c r="D29" s="0" t="n"/>
+      <c r="E29" s="80" t="n"/>
+    </row>
+    <row r="30" s="106">
+      <c r="A30" s="76" t="inlineStr">
+        <is>
+          <t>ACPP-iPhone 套數</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n"/>
+      <c r="C30" s="0" t="n"/>
+      <c r="D30" s="0" t="n"/>
+      <c r="E30" s="80" t="n"/>
+    </row>
+    <row r="31" s="106">
+      <c r="A31" s="76" t="inlineStr">
         <is>
           <t>SA Care for iPhone 套數</t>
         </is>
       </c>
-      <c r="B26" s="0" t="n">
-        <v>162</v>
-      </c>
-      <c r="C26" s="0" t="n">
-        <v>175</v>
-      </c>
-      <c r="D26" s="0" t="n">
-        <v>13</v>
-      </c>
-      <c r="E26" s="80" t="n">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="81" t="inlineStr">
-        <is>
-          <t>SA Care for iPhone 搭售率</t>
-        </is>
-      </c>
-      <c r="B27" s="87" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="C27" s="82" t="n">
-        <v>0.2709</v>
-      </c>
-      <c r="D27" s="87" t="n">
-        <v>-0.09</v>
-      </c>
-      <c r="E27" s="83" t="n">
-        <v>-0.25</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="76" t="inlineStr">
+      <c r="B31" s="0" t="n"/>
+      <c r="C31" s="0" t="n"/>
+      <c r="D31" s="0" t="n"/>
+      <c r="E31" s="80" t="n"/>
+    </row>
+    <row r="32" s="106">
+      <c r="A32" s="81" t="inlineStr">
+        <is>
+          <t>保固加總 iPhone 搭售率</t>
+        </is>
+      </c>
+      <c r="B32" s="87" t="n"/>
+      <c r="C32" s="87" t="n"/>
+      <c r="D32" s="87" t="n"/>
+      <c r="E32" s="83" t="n"/>
+    </row>
+    <row r="33" s="106">
+      <c r="A33" s="76" t="inlineStr">
         <is>
           <t>Watch 台數</t>
         </is>
       </c>
-      <c r="B28" s="0" t="n">
-        <v>199</v>
-      </c>
-      <c r="C28" s="0" t="n">
-        <v>211</v>
-      </c>
-      <c r="D28" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="E28" s="80" t="n">
-        <v>0.06</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="76" t="inlineStr">
+      <c r="B33" s="0" t="n"/>
+      <c r="C33" s="0" t="n"/>
+      <c r="D33" s="0" t="n"/>
+      <c r="E33" s="80" t="n"/>
+    </row>
+    <row r="34" s="106">
+      <c r="A34" s="76" t="inlineStr">
+        <is>
+          <t>ACPP-Watch 套數</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n"/>
+      <c r="C34" s="0" t="n"/>
+      <c r="D34" s="0" t="n"/>
+      <c r="E34" s="80" t="n"/>
+    </row>
+    <row r="35" s="106">
+      <c r="A35" s="76" t="inlineStr">
         <is>
           <t>SA Care for Watch 套數</t>
         </is>
       </c>
-      <c r="B29" s="0" t="n">
-        <v>84</v>
-      </c>
-      <c r="C29" s="0" t="n">
-        <v>92</v>
-      </c>
-      <c r="D29" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="E29" s="80" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="81" t="inlineStr">
-        <is>
-          <t>SA Care for Watch 搭售率</t>
-        </is>
-      </c>
-      <c r="B30" s="87" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="C30" s="87" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="D30" s="87" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="E30" s="83" t="n">
-        <v>0.04</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="76" t="inlineStr">
+      <c r="B35" s="0" t="n"/>
+      <c r="C35" s="0" t="n"/>
+      <c r="D35" s="0" t="n"/>
+      <c r="E35" s="80" t="n"/>
+    </row>
+    <row r="36" s="106">
+      <c r="A36" s="81" t="inlineStr">
+        <is>
+          <t>保固加總 Watch 搭售率</t>
+        </is>
+      </c>
+      <c r="B36" s="87" t="n"/>
+      <c r="C36" s="87" t="n"/>
+      <c r="D36" s="87" t="n"/>
+      <c r="E36" s="83" t="n"/>
+    </row>
+    <row r="37" s="106">
+      <c r="A37" s="76" t="inlineStr">
+        <is>
+          <t>AirPods 台數</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n"/>
+      <c r="C37" s="0" t="n"/>
+      <c r="D37" s="0" t="n"/>
+      <c r="E37" s="80" t="n"/>
+    </row>
+    <row r="38" s="106">
+      <c r="A38" s="76" t="inlineStr">
+        <is>
+          <t>ACPP-AirPods 套數</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n"/>
+      <c r="C38" s="0" t="n"/>
+      <c r="D38" s="0" t="n"/>
+      <c r="E38" s="80" t="n"/>
+    </row>
+    <row r="39" s="106">
+      <c r="A39" s="76" t="inlineStr">
+        <is>
+          <t>SA Care for AirPods 套數</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n"/>
+      <c r="C39" s="0" t="n"/>
+      <c r="D39" s="0" t="n"/>
+      <c r="E39" s="80" t="n"/>
+    </row>
+    <row r="40" s="106">
+      <c r="A40" s="81" t="inlineStr">
+        <is>
+          <t>保固加總 AirPods 搭售率</t>
+        </is>
+      </c>
+      <c r="B40" s="87" t="n"/>
+      <c r="C40" s="87" t="n"/>
+      <c r="D40" s="87" t="n"/>
+      <c r="E40" s="83" t="n"/>
+    </row>
+    <row r="41" s="106">
+      <c r="A41" s="76" t="inlineStr">
         <is>
           <t>人均產值</t>
         </is>
       </c>
-      <c r="B31" s="77" t="n"/>
-      <c r="C31" s="77" t="n"/>
-      <c r="D31" s="77" t="n"/>
-      <c r="E31" s="80" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="76" t="inlineStr">
+      <c r="B41" s="77" t="n"/>
+      <c r="C41" s="77" t="n"/>
+      <c r="D41" s="77" t="n"/>
+      <c r="E41" s="80" t="n"/>
+    </row>
+    <row r="42" s="106">
+      <c r="A42" s="76" t="inlineStr">
         <is>
           <t>來客數</t>
         </is>
       </c>
-      <c r="B32" s="77" t="n"/>
-      <c r="C32" s="77" t="n"/>
-      <c r="E32" s="80" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="84" t="inlineStr">
+      <c r="B42" s="77" t="n"/>
+      <c r="C42" s="77" t="n"/>
+      <c r="E42" s="80" t="n"/>
+    </row>
+    <row r="43" s="106">
+      <c r="A43" s="84" t="inlineStr">
         <is>
           <t>成交筆數</t>
         </is>
       </c>
-      <c r="B33" s="74" t="n"/>
-      <c r="C33" s="74" t="n"/>
-      <c r="D33" s="73" t="n"/>
-      <c r="E33" s="85" t="n"/>
-    </row>
-    <row r="34">
-      <c r="B34" s="71" t="n"/>
-      <c r="C34" s="71" t="n"/>
+      <c r="B43" s="74" t="n"/>
+      <c r="C43" s="74" t="n"/>
+      <c r="D43" s="73" t="n"/>
+      <c r="E43" s="85" t="n"/>
+    </row>
+    <row r="44" s="106">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>提袋率</t>
+        </is>
+      </c>
+      <c r="B44" s="71" t="n"/>
+      <c r="C44" s="71" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6526,7 +6418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:P43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="31" bestFit="1" customWidth="1" style="106" min="1" max="1"/>
@@ -6859,11 +6751,11 @@
     <row r="13" ht="17" customHeight="1" s="106">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>AirPods Max</t>
-        </is>
-      </c>
-      <c r="B13" s="17" t="n"/>
-      <c r="C13" s="17" t="n"/>
+          <t>AirPods 5</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="16" t="n"/>
       <c r="D13" s="17" t="n"/>
       <c r="E13" s="17" t="n"/>
       <c r="F13" s="17" t="n"/>
@@ -6881,7 +6773,7 @@
     <row r="14" ht="17" customHeight="1" s="106">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>HomePod MIni</t>
+          <t>AirPods Max</t>
         </is>
       </c>
       <c r="B14" s="17" t="n"/>
@@ -6903,7 +6795,7 @@
     <row r="15" ht="17" customHeight="1" s="106">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>HomePod</t>
+          <t>HomePod MIni</t>
         </is>
       </c>
       <c r="B15" s="17" t="n"/>
@@ -6923,57 +6815,57 @@
       <c r="P15" s="18" t="n"/>
     </row>
     <row r="16" ht="17" customHeight="1" s="106">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>HomePod</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="17" t="n"/>
+      <c r="H16" s="17" t="n"/>
+      <c r="I16" s="17" t="n"/>
+      <c r="J16" s="17" t="n"/>
+      <c r="K16" s="17" t="n"/>
+      <c r="L16" s="17" t="n"/>
+      <c r="M16" s="17" t="n"/>
+      <c r="N16" s="17" t="n"/>
+      <c r="O16" s="17" t="n"/>
+      <c r="P16" s="18" t="n"/>
+    </row>
+    <row r="17" ht="17" customHeight="1" s="106">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>音頻合計</t>
         </is>
       </c>
-      <c r="B16" s="19" t="n"/>
-      <c r="C16" s="19" t="n"/>
-      <c r="D16" s="19" t="n"/>
-      <c r="E16" s="19" t="n"/>
-      <c r="F16" s="19" t="n"/>
-      <c r="G16" s="19" t="n"/>
-      <c r="H16" s="19" t="n"/>
-      <c r="I16" s="19" t="n"/>
-      <c r="J16" s="19" t="n"/>
-      <c r="K16" s="19" t="n"/>
-      <c r="L16" s="19" t="n"/>
-      <c r="M16" s="19" t="n"/>
-      <c r="N16" s="19" t="n"/>
-      <c r="O16" s="19" t="n"/>
-      <c r="P16" s="19" t="n"/>
-    </row>
-    <row r="17" ht="17" customHeight="1" s="106">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>AppleWatch S11</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="n"/>
-      <c r="C17" s="16" t="n"/>
-      <c r="D17" s="17" t="n"/>
-      <c r="E17" s="17" t="n"/>
-      <c r="F17" s="17" t="n"/>
-      <c r="G17" s="17" t="n"/>
-      <c r="H17" s="17" t="n"/>
-      <c r="I17" s="17" t="n"/>
-      <c r="J17" s="17" t="n"/>
-      <c r="K17" s="17" t="n"/>
-      <c r="L17" s="17" t="n"/>
-      <c r="M17" s="17" t="n"/>
-      <c r="N17" s="17" t="n"/>
-      <c r="O17" s="17" t="n"/>
-      <c r="P17" s="18" t="n"/>
+      <c r="B17" s="19" t="n"/>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="n"/>
+      <c r="H17" s="19" t="n"/>
+      <c r="I17" s="19" t="n"/>
+      <c r="J17" s="19" t="n"/>
+      <c r="K17" s="19" t="n"/>
+      <c r="L17" s="19" t="n"/>
+      <c r="M17" s="19" t="n"/>
+      <c r="N17" s="19" t="n"/>
+      <c r="O17" s="19" t="n"/>
+      <c r="P17" s="19" t="n"/>
     </row>
     <row r="18" ht="17" customHeight="1" s="106">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>AppleWatch Ultra 3</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="n"/>
-      <c r="C18" s="17" t="n"/>
+          <t>AppleWatch S11</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="n"/>
+      <c r="C18" s="16" t="n"/>
       <c r="D18" s="17" t="n"/>
       <c r="E18" s="17" t="n"/>
       <c r="F18" s="17" t="n"/>
@@ -6991,7 +6883,7 @@
     <row r="19" ht="17" customHeight="1" s="106">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>AppleWatch SE3</t>
+          <t>AppleWatch S12</t>
         </is>
       </c>
       <c r="B19" s="16" t="n"/>
@@ -7011,35 +6903,35 @@
       <c r="P19" s="18" t="n"/>
     </row>
     <row r="20" ht="17" customHeight="1" s="106">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>AppleWatch 合計</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="n"/>
-      <c r="C20" s="19" t="n"/>
-      <c r="D20" s="19" t="n"/>
-      <c r="E20" s="19" t="n"/>
-      <c r="F20" s="19" t="n"/>
-      <c r="G20" s="19" t="n"/>
-      <c r="H20" s="19" t="n"/>
-      <c r="I20" s="19" t="n"/>
-      <c r="J20" s="19" t="n"/>
-      <c r="K20" s="19" t="n"/>
-      <c r="L20" s="19" t="n"/>
-      <c r="M20" s="19" t="n"/>
-      <c r="N20" s="19" t="n"/>
-      <c r="O20" s="19" t="n"/>
-      <c r="P20" s="19" t="n"/>
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>AppleWatch Ultra 3</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="17" t="n"/>
+      <c r="G20" s="17" t="n"/>
+      <c r="H20" s="17" t="n"/>
+      <c r="I20" s="17" t="n"/>
+      <c r="J20" s="17" t="n"/>
+      <c r="K20" s="17" t="n"/>
+      <c r="L20" s="17" t="n"/>
+      <c r="M20" s="17" t="n"/>
+      <c r="N20" s="17" t="n"/>
+      <c r="O20" s="17" t="n"/>
+      <c r="P20" s="18" t="n"/>
     </row>
     <row r="21" ht="17" customHeight="1" s="106">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>iPhone 17</t>
-        </is>
-      </c>
-      <c r="B21" s="16" t="n"/>
-      <c r="C21" s="16" t="n"/>
+          <t>AppleWatch Ultra 4</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="n"/>
+      <c r="C21" s="17" t="n"/>
       <c r="D21" s="17" t="n"/>
       <c r="E21" s="17" t="n"/>
       <c r="F21" s="17" t="n"/>
@@ -7057,11 +6949,11 @@
     <row r="22" ht="17" customHeight="1" s="106">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>iPhone Air</t>
-        </is>
-      </c>
-      <c r="B22" s="17" t="n"/>
-      <c r="C22" s="17" t="n"/>
+          <t>AppleWatch SE3</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="n"/>
+      <c r="C22" s="16" t="n"/>
       <c r="D22" s="17" t="n"/>
       <c r="E22" s="17" t="n"/>
       <c r="F22" s="17" t="n"/>
@@ -7077,31 +6969,31 @@
       <c r="P22" s="18" t="n"/>
     </row>
     <row r="23" ht="17" customHeight="1" s="106">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>iPhone 17 Pro</t>
-        </is>
-      </c>
-      <c r="B23" s="16" t="n"/>
-      <c r="C23" s="16" t="n"/>
-      <c r="D23" s="17" t="n"/>
-      <c r="E23" s="17" t="n"/>
-      <c r="F23" s="17" t="n"/>
-      <c r="G23" s="17" t="n"/>
-      <c r="H23" s="17" t="n"/>
-      <c r="I23" s="17" t="n"/>
-      <c r="J23" s="17" t="n"/>
-      <c r="K23" s="17" t="n"/>
-      <c r="L23" s="17" t="n"/>
-      <c r="M23" s="17" t="n"/>
-      <c r="N23" s="17" t="n"/>
-      <c r="O23" s="17" t="n"/>
-      <c r="P23" s="18" t="n"/>
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>AppleWatch 合計</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="n"/>
+      <c r="C23" s="19" t="n"/>
+      <c r="D23" s="19" t="n"/>
+      <c r="E23" s="19" t="n"/>
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="19" t="n"/>
+      <c r="H23" s="19" t="n"/>
+      <c r="I23" s="19" t="n"/>
+      <c r="J23" s="19" t="n"/>
+      <c r="K23" s="19" t="n"/>
+      <c r="L23" s="19" t="n"/>
+      <c r="M23" s="19" t="n"/>
+      <c r="N23" s="19" t="n"/>
+      <c r="O23" s="19" t="n"/>
+      <c r="P23" s="19" t="n"/>
     </row>
     <row r="24" ht="17" customHeight="1" s="106">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>iPhone 17 Pro Max</t>
+          <t>iPhone 17</t>
         </is>
       </c>
       <c r="B24" s="16" t="n"/>
@@ -7123,11 +7015,11 @@
     <row r="25" ht="17" customHeight="1" s="106">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>iPhone 17e</t>
-        </is>
-      </c>
-      <c r="B25" s="16" t="n"/>
-      <c r="C25" s="16" t="n"/>
+          <t>iPhone Air</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="n"/>
+      <c r="C25" s="17" t="n"/>
       <c r="D25" s="17" t="n"/>
       <c r="E25" s="17" t="n"/>
       <c r="F25" s="17" t="n"/>
@@ -7143,31 +7035,31 @@
       <c r="P25" s="18" t="n"/>
     </row>
     <row r="26" ht="17" customHeight="1" s="106">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>iPhone 合計</t>
-        </is>
-      </c>
-      <c r="B26" s="19" t="n"/>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="19" t="n"/>
-      <c r="E26" s="19" t="n"/>
-      <c r="F26" s="19" t="n"/>
-      <c r="G26" s="19" t="n"/>
-      <c r="H26" s="19" t="n"/>
-      <c r="I26" s="19" t="n"/>
-      <c r="J26" s="19" t="n"/>
-      <c r="K26" s="19" t="n"/>
-      <c r="L26" s="19" t="n"/>
-      <c r="M26" s="19" t="n"/>
-      <c r="N26" s="19" t="n"/>
-      <c r="O26" s="19" t="n"/>
-      <c r="P26" s="19" t="n"/>
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>iPhone 17 Pro</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="n"/>
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="17" t="n"/>
+      <c r="E26" s="17" t="n"/>
+      <c r="F26" s="17" t="n"/>
+      <c r="G26" s="17" t="n"/>
+      <c r="H26" s="17" t="n"/>
+      <c r="I26" s="17" t="n"/>
+      <c r="J26" s="17" t="n"/>
+      <c r="K26" s="17" t="n"/>
+      <c r="L26" s="17" t="n"/>
+      <c r="M26" s="17" t="n"/>
+      <c r="N26" s="17" t="n"/>
+      <c r="O26" s="17" t="n"/>
+      <c r="P26" s="18" t="n"/>
     </row>
     <row r="27" ht="17" customHeight="1" s="106">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>iPad A16</t>
+          <t>iPhone 17 Pro Max</t>
         </is>
       </c>
       <c r="B27" s="16" t="n"/>
@@ -7189,10 +7081,10 @@
     <row r="28" ht="17" customHeight="1" s="106">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>iPad Air 11</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="n"/>
+          <t>iPhone 17e</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="n"/>
       <c r="C28" s="16" t="n"/>
       <c r="D28" s="17" t="n"/>
       <c r="E28" s="17" t="n"/>
@@ -7211,10 +7103,10 @@
     <row r="29" ht="17" customHeight="1" s="106">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>iPad Air 13</t>
-        </is>
-      </c>
-      <c r="B29" s="17" t="n"/>
+          <t>iPhone 18 Pro</t>
+        </is>
+      </c>
+      <c r="B29" s="16" t="n"/>
       <c r="C29" s="16" t="n"/>
       <c r="D29" s="17" t="n"/>
       <c r="E29" s="17" t="n"/>
@@ -7233,7 +7125,7 @@
     <row r="30" ht="17" customHeight="1" s="106">
       <c r="A30" s="16" t="inlineStr">
         <is>
-          <t>iPad Pro 11 M5</t>
+          <t>iPhone 18 Pro Max</t>
         </is>
       </c>
       <c r="B30" s="16" t="n"/>
@@ -7253,31 +7145,31 @@
       <c r="P30" s="18" t="n"/>
     </row>
     <row r="31" ht="17" customHeight="1" s="106">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>iPad Pro 13 M5</t>
-        </is>
-      </c>
-      <c r="B31" s="16" t="n"/>
-      <c r="C31" s="17" t="n"/>
-      <c r="D31" s="17" t="n"/>
-      <c r="E31" s="17" t="n"/>
-      <c r="F31" s="17" t="n"/>
-      <c r="G31" s="17" t="n"/>
-      <c r="H31" s="17" t="n"/>
-      <c r="I31" s="17" t="n"/>
-      <c r="J31" s="17" t="n"/>
-      <c r="K31" s="17" t="n"/>
-      <c r="L31" s="17" t="n"/>
-      <c r="M31" s="17" t="n"/>
-      <c r="N31" s="17" t="n"/>
-      <c r="O31" s="17" t="n"/>
-      <c r="P31" s="18" t="n"/>
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>iPhone 合計</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="n"/>
+      <c r="C31" s="19" t="n"/>
+      <c r="D31" s="19" t="n"/>
+      <c r="E31" s="19" t="n"/>
+      <c r="F31" s="19" t="n"/>
+      <c r="G31" s="19" t="n"/>
+      <c r="H31" s="19" t="n"/>
+      <c r="I31" s="19" t="n"/>
+      <c r="J31" s="19" t="n"/>
+      <c r="K31" s="19" t="n"/>
+      <c r="L31" s="19" t="n"/>
+      <c r="M31" s="19" t="n"/>
+      <c r="N31" s="19" t="n"/>
+      <c r="O31" s="19" t="n"/>
+      <c r="P31" s="19" t="n"/>
     </row>
     <row r="32" ht="17" customHeight="1" s="106">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t>iPad mini</t>
+          <t>iPad A16</t>
         </is>
       </c>
       <c r="B32" s="16" t="n"/>
@@ -7297,35 +7189,35 @@
       <c r="P32" s="18" t="n"/>
     </row>
     <row r="33" ht="17" customHeight="1" s="106">
-      <c r="A33" s="19" t="inlineStr">
-        <is>
-          <t>iPad 合計</t>
-        </is>
-      </c>
-      <c r="B33" s="19" t="n"/>
-      <c r="C33" s="19" t="n"/>
-      <c r="D33" s="19" t="n"/>
-      <c r="E33" s="19" t="n"/>
-      <c r="F33" s="19" t="n"/>
-      <c r="G33" s="19" t="n"/>
-      <c r="H33" s="19" t="n"/>
-      <c r="I33" s="19" t="n"/>
-      <c r="J33" s="19" t="n"/>
-      <c r="K33" s="19" t="n"/>
-      <c r="L33" s="19" t="n"/>
-      <c r="M33" s="19" t="n"/>
-      <c r="N33" s="19" t="n"/>
-      <c r="O33" s="19" t="n"/>
-      <c r="P33" s="19" t="n"/>
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>iPad Air 11</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="16" t="n"/>
+      <c r="D33" s="17" t="n"/>
+      <c r="E33" s="17" t="n"/>
+      <c r="F33" s="17" t="n"/>
+      <c r="G33" s="17" t="n"/>
+      <c r="H33" s="17" t="n"/>
+      <c r="I33" s="17" t="n"/>
+      <c r="J33" s="17" t="n"/>
+      <c r="K33" s="17" t="n"/>
+      <c r="L33" s="17" t="n"/>
+      <c r="M33" s="17" t="n"/>
+      <c r="N33" s="17" t="n"/>
+      <c r="O33" s="17" t="n"/>
+      <c r="P33" s="18" t="n"/>
     </row>
     <row r="34" ht="17" customHeight="1" s="106">
       <c r="A34" s="16" t="inlineStr">
         <is>
-          <t>Apple Pencil 第一代</t>
+          <t>iPad Air 13</t>
         </is>
       </c>
       <c r="B34" s="17" t="n"/>
-      <c r="C34" s="17" t="n"/>
+      <c r="C34" s="16" t="n"/>
       <c r="D34" s="17" t="n"/>
       <c r="E34" s="17" t="n"/>
       <c r="F34" s="17" t="n"/>
@@ -7343,11 +7235,11 @@
     <row r="35" ht="17" customHeight="1" s="106">
       <c r="A35" s="16" t="inlineStr">
         <is>
-          <t>Apple Pencil 第二代</t>
-        </is>
-      </c>
-      <c r="B35" s="17" t="n"/>
-      <c r="C35" s="17" t="n"/>
+          <t>iPad Pro 11 M5</t>
+        </is>
+      </c>
+      <c r="B35" s="16" t="n"/>
+      <c r="C35" s="16" t="n"/>
       <c r="D35" s="17" t="n"/>
       <c r="E35" s="17" t="n"/>
       <c r="F35" s="17" t="n"/>
@@ -7365,11 +7257,11 @@
     <row r="36" ht="17" customHeight="1" s="106">
       <c r="A36" s="16" t="inlineStr">
         <is>
-          <t>Apple Pencil (USB-C)</t>
+          <t>iPad Pro 13 M5</t>
         </is>
       </c>
       <c r="B36" s="16" t="n"/>
-      <c r="C36" s="16" t="n"/>
+      <c r="C36" s="17" t="n"/>
       <c r="D36" s="17" t="n"/>
       <c r="E36" s="17" t="n"/>
       <c r="F36" s="17" t="n"/>
@@ -7387,7 +7279,7 @@
     <row r="37" ht="17" customHeight="1" s="106">
       <c r="A37" s="16" t="inlineStr">
         <is>
-          <t>Apple Pencil Pro</t>
+          <t>iPad mini</t>
         </is>
       </c>
       <c r="B37" s="16" t="n"/>
@@ -7409,7 +7301,7 @@
     <row r="38" ht="17" customHeight="1" s="106">
       <c r="A38" s="19" t="inlineStr">
         <is>
-          <t>Apple Pencil 合計</t>
+          <t>iPad 合計</t>
         </is>
       </c>
       <c r="B38" s="19" t="n"/>
@@ -7427,6 +7319,116 @@
       <c r="N38" s="19" t="n"/>
       <c r="O38" s="19" t="n"/>
       <c r="P38" s="19" t="n"/>
+    </row>
+    <row r="39" ht="17" customHeight="1" s="106">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>Apple Pencil 第一代</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="n"/>
+      <c r="C39" s="17" t="n"/>
+      <c r="D39" s="17" t="n"/>
+      <c r="E39" s="17" t="n"/>
+      <c r="F39" s="17" t="n"/>
+      <c r="G39" s="17" t="n"/>
+      <c r="H39" s="17" t="n"/>
+      <c r="I39" s="17" t="n"/>
+      <c r="J39" s="17" t="n"/>
+      <c r="K39" s="17" t="n"/>
+      <c r="L39" s="17" t="n"/>
+      <c r="M39" s="17" t="n"/>
+      <c r="N39" s="17" t="n"/>
+      <c r="O39" s="17" t="n"/>
+      <c r="P39" s="18" t="n"/>
+    </row>
+    <row r="40" ht="17" customHeight="1" s="106">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>Apple Pencil 第二代</t>
+        </is>
+      </c>
+      <c r="B40" s="17" t="n"/>
+      <c r="C40" s="17" t="n"/>
+      <c r="D40" s="17" t="n"/>
+      <c r="E40" s="17" t="n"/>
+      <c r="F40" s="17" t="n"/>
+      <c r="G40" s="17" t="n"/>
+      <c r="H40" s="17" t="n"/>
+      <c r="I40" s="17" t="n"/>
+      <c r="J40" s="17" t="n"/>
+      <c r="K40" s="17" t="n"/>
+      <c r="L40" s="17" t="n"/>
+      <c r="M40" s="17" t="n"/>
+      <c r="N40" s="17" t="n"/>
+      <c r="O40" s="17" t="n"/>
+      <c r="P40" s="18" t="n"/>
+    </row>
+    <row r="41" ht="17" customHeight="1" s="106">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>Apple Pencil (USB-C)</t>
+        </is>
+      </c>
+      <c r="B41" s="16" t="n"/>
+      <c r="C41" s="16" t="n"/>
+      <c r="D41" s="17" t="n"/>
+      <c r="E41" s="17" t="n"/>
+      <c r="F41" s="17" t="n"/>
+      <c r="G41" s="17" t="n"/>
+      <c r="H41" s="17" t="n"/>
+      <c r="I41" s="17" t="n"/>
+      <c r="J41" s="17" t="n"/>
+      <c r="K41" s="17" t="n"/>
+      <c r="L41" s="17" t="n"/>
+      <c r="M41" s="17" t="n"/>
+      <c r="N41" s="17" t="n"/>
+      <c r="O41" s="17" t="n"/>
+      <c r="P41" s="18" t="n"/>
+    </row>
+    <row r="42" ht="17" customHeight="1" s="106">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>Apple Pencil Pro</t>
+        </is>
+      </c>
+      <c r="B42" s="16" t="n"/>
+      <c r="C42" s="16" t="n"/>
+      <c r="D42" s="17" t="n"/>
+      <c r="E42" s="17" t="n"/>
+      <c r="F42" s="17" t="n"/>
+      <c r="G42" s="17" t="n"/>
+      <c r="H42" s="17" t="n"/>
+      <c r="I42" s="17" t="n"/>
+      <c r="J42" s="17" t="n"/>
+      <c r="K42" s="17" t="n"/>
+      <c r="L42" s="17" t="n"/>
+      <c r="M42" s="17" t="n"/>
+      <c r="N42" s="17" t="n"/>
+      <c r="O42" s="17" t="n"/>
+      <c r="P42" s="18" t="n"/>
+    </row>
+    <row r="43" ht="17" customHeight="1" s="106">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>Apple Pencil 合計</t>
+        </is>
+      </c>
+      <c r="B43" s="19" t="n"/>
+      <c r="C43" s="19" t="n"/>
+      <c r="D43" s="19" t="n"/>
+      <c r="E43" s="19" t="n"/>
+      <c r="F43" s="19" t="n"/>
+      <c r="G43" s="19" t="n"/>
+      <c r="H43" s="19" t="n"/>
+      <c r="I43" s="19" t="n"/>
+      <c r="J43" s="19" t="n"/>
+      <c r="K43" s="19" t="n"/>
+      <c r="L43" s="19" t="n"/>
+      <c r="M43" s="19" t="n"/>
+      <c r="N43" s="19" t="n"/>
+      <c r="O43" s="19" t="n"/>
+      <c r="P43" s="19" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8549,7 +8551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="29.1640625" customWidth="1" style="106" min="1" max="1"/>
@@ -8634,1233 +8636,627 @@
     <row r="2" ht="34" customHeight="1" s="106">
       <c r="A2" s="20" t="inlineStr">
         <is>
-          <t>總營業額</t>
-        </is>
-      </c>
-      <c r="B2" s="29" t="n">
-        <v>1246331</v>
-      </c>
-      <c r="C2" s="29" t="n">
-        <v>1683829</v>
-      </c>
-      <c r="D2" s="30" t="n">
-        <v>-266354</v>
-      </c>
-      <c r="E2" s="31" t="n">
-        <v>-0.11</v>
-      </c>
-      <c r="F2" s="29" t="n">
-        <v>2930160</v>
-      </c>
+          <t>總營業額(a + c + d + e)</t>
+        </is>
+      </c>
+      <c r="B2" s="29" t="n"/>
+      <c r="C2" s="29" t="n"/>
+      <c r="D2" s="30" t="n"/>
+      <c r="E2" s="31" t="n"/>
+      <c r="F2" s="29" t="n"/>
       <c r="G2" s="110" t="n"/>
-      <c r="H2" s="31" t="n">
-        <v>1.1</v>
-      </c>
+      <c r="H2" s="31" t="n"/>
       <c r="I2" s="29" t="n"/>
-      <c r="J2" s="30" t="n">
-        <v>-4764080</v>
-      </c>
-      <c r="K2" s="31" t="n">
-        <v>-0.33</v>
-      </c>
-      <c r="L2" s="29" t="n">
-        <v>2728236</v>
-      </c>
-      <c r="M2" s="30" t="n">
-        <v>1696122</v>
-      </c>
-      <c r="N2" s="31" t="n">
-        <v>0.21</v>
-      </c>
+      <c r="J2" s="30" t="n"/>
+      <c r="K2" s="31" t="n"/>
+      <c r="L2" s="29" t="n"/>
+      <c r="M2" s="30" t="n"/>
+      <c r="N2" s="31" t="n"/>
     </row>
     <row r="3" ht="34" customHeight="1" s="106">
       <c r="A3" s="20" t="inlineStr">
         <is>
-          <t>零售營業額</t>
-        </is>
-      </c>
-      <c r="B3" s="29" t="n">
-        <v>1246331</v>
-      </c>
-      <c r="C3" s="29" t="n">
-        <v>1683829</v>
-      </c>
-      <c r="D3" s="30" t="n">
-        <v>-266354</v>
-      </c>
-      <c r="E3" s="31" t="n">
-        <v>-0.11</v>
-      </c>
-      <c r="F3" s="29" t="n">
-        <v>2930160</v>
-      </c>
+          <t>零售營業額(a)</t>
+        </is>
+      </c>
+      <c r="B3" s="29" t="n"/>
+      <c r="C3" s="29" t="n"/>
+      <c r="D3" s="30" t="n"/>
+      <c r="E3" s="31" t="n"/>
+      <c r="F3" s="29" t="n"/>
       <c r="G3" s="110" t="n"/>
-      <c r="H3" s="31" t="n">
-        <v>1.1</v>
-      </c>
+      <c r="H3" s="31" t="n"/>
       <c r="I3" s="29" t="n"/>
-      <c r="J3" s="30" t="n">
-        <v>-4764080</v>
-      </c>
-      <c r="K3" s="31" t="n">
-        <v>-0.33</v>
-      </c>
-      <c r="L3" s="29" t="n">
-        <v>2728236</v>
-      </c>
-      <c r="M3" s="30" t="n">
-        <v>1696122</v>
-      </c>
-      <c r="N3" s="31" t="n">
-        <v>0.21</v>
-      </c>
+      <c r="J3" s="30" t="n"/>
+      <c r="K3" s="31" t="n"/>
+      <c r="L3" s="29" t="n"/>
+      <c r="M3" s="30" t="n"/>
+      <c r="N3" s="31" t="n"/>
     </row>
     <row r="4" ht="34" customHeight="1" s="106">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t>專案營業額</t>
+          <t>訂單出貨金額(b)</t>
         </is>
       </c>
       <c r="B4" s="29" t="n"/>
       <c r="C4" s="29" t="n"/>
-      <c r="D4" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" s="32" t="n"/>
+      <c r="D4" s="30" t="n"/>
+      <c r="E4" s="31" t="n"/>
       <c r="F4" s="29" t="n"/>
       <c r="G4" s="110" t="n"/>
-      <c r="H4" s="31" t="n">
-        <v>0</v>
-      </c>
+      <c r="H4" s="31" t="n"/>
       <c r="I4" s="29" t="n"/>
-      <c r="J4" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K4" s="32" t="n"/>
+      <c r="J4" s="30" t="n"/>
+      <c r="K4" s="31" t="n"/>
       <c r="L4" s="29" t="n"/>
-      <c r="M4" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N4" s="32" t="n"/>
+      <c r="M4" s="30" t="n"/>
+      <c r="N4" s="31" t="n"/>
     </row>
     <row r="5" ht="34" customHeight="1" s="106">
       <c r="A5" s="20" t="inlineStr">
         <is>
-          <t>Apple 主機營業額</t>
-        </is>
-      </c>
-      <c r="B5" s="29" t="n">
-        <v>1002000</v>
-      </c>
-      <c r="C5" s="29" t="n">
-        <v>1230590</v>
-      </c>
-      <c r="D5" s="30" t="n">
-        <v>-254958</v>
-      </c>
-      <c r="E5" s="31" t="n">
-        <v>-0.14</v>
-      </c>
-      <c r="F5" s="29" t="n">
-        <v>2232590</v>
-      </c>
+          <t>當日零售營業收入(a + b)</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="n"/>
+      <c r="C5" s="29" t="n"/>
+      <c r="D5" s="30" t="n"/>
+      <c r="E5" s="31" t="n"/>
+      <c r="F5" s="29" t="n"/>
       <c r="G5" s="110" t="n"/>
-      <c r="H5" s="31" t="n">
-        <v>1.12</v>
-      </c>
+      <c r="H5" s="31" t="n"/>
       <c r="I5" s="29" t="n"/>
-      <c r="J5" s="30" t="n">
-        <v>-4081504</v>
-      </c>
-      <c r="K5" s="31" t="n">
-        <v>-0.36</v>
-      </c>
-      <c r="L5" s="29" t="n">
-        <v>2085085</v>
-      </c>
-      <c r="M5" s="30" t="n">
-        <v>1392318</v>
-      </c>
-      <c r="N5" s="31" t="n">
-        <v>0.24</v>
-      </c>
+      <c r="J5" s="30" t="n"/>
+      <c r="K5" s="31" t="n"/>
+      <c r="L5" s="29" t="n"/>
+      <c r="M5" s="30" t="n"/>
+      <c r="N5" s="31" t="n"/>
     </row>
     <row r="6" ht="34" customHeight="1" s="106">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>Apple 配件營業額</t>
-        </is>
-      </c>
-      <c r="B6" s="29" t="n">
-        <v>81630</v>
-      </c>
-      <c r="C6" s="29" t="n">
-        <v>164871</v>
-      </c>
-      <c r="D6" s="30" t="n">
-        <v>-17290</v>
-      </c>
-      <c r="E6" s="31" t="n">
-        <v>-0.11</v>
-      </c>
-      <c r="F6" s="29" t="n">
-        <v>246501</v>
-      </c>
+          <t>零售訂金營業額(c)</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="n"/>
+      <c r="C6" s="29" t="n"/>
+      <c r="D6" s="30" t="n"/>
+      <c r="E6" s="31" t="n"/>
+      <c r="F6" s="29" t="n"/>
       <c r="G6" s="110" t="n"/>
-      <c r="H6" s="31" t="n">
-        <v>0.77</v>
-      </c>
+      <c r="H6" s="31" t="n"/>
       <c r="I6" s="29" t="n"/>
-      <c r="J6" s="30" t="n">
-        <v>-397539</v>
-      </c>
-      <c r="K6" s="31" t="n">
-        <v>-0.29</v>
-      </c>
-      <c r="L6" s="29" t="n">
-        <v>287551</v>
-      </c>
-      <c r="M6" s="30" t="n">
-        <v>-125359</v>
-      </c>
-      <c r="N6" s="31" t="n">
-        <v>-0.11</v>
-      </c>
+      <c r="J6" s="30" t="n"/>
+      <c r="K6" s="31" t="n"/>
+      <c r="L6" s="29" t="n"/>
+      <c r="M6" s="30" t="n"/>
+      <c r="N6" s="31" t="n"/>
     </row>
     <row r="7" ht="34" customHeight="1" s="106">
       <c r="A7" s="20" t="inlineStr">
         <is>
-          <t>3PP配件營業額</t>
-        </is>
-      </c>
-      <c r="B7" s="29" t="n">
-        <v>114151</v>
-      </c>
-      <c r="C7" s="29" t="n">
-        <v>222248</v>
-      </c>
-      <c r="D7" s="30" t="n">
-        <v>17294</v>
-      </c>
-      <c r="E7" s="31" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F7" s="29" t="n">
-        <v>336399</v>
-      </c>
+          <t>專案營業額(d)</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="n"/>
+      <c r="C7" s="29" t="n"/>
+      <c r="D7" s="30" t="n"/>
+      <c r="E7" s="32" t="n"/>
+      <c r="F7" s="29" t="n"/>
       <c r="G7" s="110" t="n"/>
-      <c r="H7" s="31" t="n">
-        <v>1.46</v>
-      </c>
+      <c r="H7" s="31" t="n"/>
       <c r="I7" s="29" t="n"/>
-      <c r="J7" s="30" t="n">
-        <v>-32577</v>
-      </c>
-      <c r="K7" s="31" t="n">
-        <v>-0.03</v>
-      </c>
-      <c r="L7" s="29" t="n">
-        <v>202150</v>
-      </c>
-      <c r="M7" s="30" t="n">
-        <v>450803</v>
-      </c>
-      <c r="N7" s="31" t="n">
-        <v>0.64</v>
-      </c>
+      <c r="J7" s="30" t="n"/>
+      <c r="K7" s="32" t="n"/>
+      <c r="L7" s="29" t="n"/>
+      <c r="M7" s="30" t="n"/>
+      <c r="N7" s="32" t="n"/>
     </row>
     <row r="8" ht="34" customHeight="1" s="106">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>3PP搭售率</t>
-        </is>
-      </c>
-      <c r="B8" s="33" t="n">
-        <v>0.0916</v>
-      </c>
-      <c r="C8" s="33" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="D8" s="33" t="n">
-        <v>0.0212</v>
-      </c>
-      <c r="E8" s="34" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="F8" s="33" t="n">
-        <v>0.1148</v>
-      </c>
-      <c r="G8" s="33" t="n"/>
-      <c r="H8" s="31" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="I8" s="33" t="n"/>
-      <c r="J8" s="33" t="n">
-        <v>0.0377</v>
-      </c>
-      <c r="K8" s="34" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="L8" s="33" t="n">
-        <v>0.0741</v>
-      </c>
-      <c r="M8" s="33" t="n">
-        <v>0.0311</v>
-      </c>
-      <c r="N8" s="34" t="n">
-        <v>0.35</v>
-      </c>
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Apple 主機營業額</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="n"/>
+      <c r="C8" s="29" t="n"/>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="31" t="n"/>
+      <c r="F8" s="29" t="n"/>
+      <c r="G8" s="110" t="n"/>
+      <c r="H8" s="31" t="n"/>
+      <c r="I8" s="29" t="n"/>
+      <c r="J8" s="30" t="n"/>
+      <c r="K8" s="31" t="n"/>
+      <c r="L8" s="29" t="n"/>
+      <c r="M8" s="30" t="n"/>
+      <c r="N8" s="31" t="n"/>
     </row>
     <row r="9" ht="34" customHeight="1" s="106">
       <c r="A9" s="20" t="inlineStr">
         <is>
-          <t>SA Care 營業額</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="n">
-        <v>48550</v>
-      </c>
-      <c r="C9" s="29" t="n">
-        <v>66120</v>
-      </c>
-      <c r="D9" s="30" t="n">
-        <v>-11400</v>
-      </c>
-      <c r="E9" s="31" t="n">
-        <v>-0.13</v>
-      </c>
-      <c r="F9" s="29" t="n">
-        <v>114670</v>
-      </c>
+          <t>Apple 配件營業額</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="n"/>
+      <c r="C9" s="29" t="n"/>
+      <c r="D9" s="30" t="n"/>
+      <c r="E9" s="31" t="n"/>
+      <c r="F9" s="29" t="n"/>
       <c r="G9" s="110" t="n"/>
-      <c r="H9" s="31" t="n">
-        <v>0.86</v>
-      </c>
+      <c r="H9" s="31" t="n"/>
       <c r="I9" s="29" t="n"/>
-      <c r="J9" s="30" t="n">
-        <v>-252460</v>
-      </c>
-      <c r="K9" s="31" t="n">
-        <v>-0.45</v>
-      </c>
-      <c r="L9" s="29" t="n">
-        <v>153450</v>
-      </c>
-      <c r="M9" s="30" t="n">
-        <v>-21640</v>
-      </c>
-      <c r="N9" s="31" t="n">
-        <v>-0.07000000000000001</v>
-      </c>
+      <c r="J9" s="30" t="n"/>
+      <c r="K9" s="31" t="n"/>
+      <c r="L9" s="29" t="n"/>
+      <c r="M9" s="30" t="n"/>
+      <c r="N9" s="31" t="n"/>
     </row>
     <row r="10" ht="34" customHeight="1" s="106">
-      <c r="A10" s="27" t="inlineStr">
-        <is>
-          <t>SA Care 搭售率</t>
-        </is>
-      </c>
-      <c r="B10" s="33" t="n">
-        <v>0.039</v>
-      </c>
-      <c r="C10" s="33" t="n">
-        <v>0.0393</v>
-      </c>
-      <c r="D10" s="33" t="n">
-        <v>-0.0008</v>
-      </c>
-      <c r="E10" s="34" t="n">
-        <v>-0.02</v>
-      </c>
-      <c r="F10" s="33" t="n">
-        <v>0.0391</v>
-      </c>
-      <c r="G10" s="33" t="n"/>
-      <c r="H10" s="31" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="I10" s="33" t="n"/>
-      <c r="J10" s="33" t="n">
-        <v>-0.007</v>
-      </c>
-      <c r="K10" s="34" t="n">
-        <v>-0.18</v>
-      </c>
-      <c r="L10" s="33" t="n">
-        <v>0.0562</v>
-      </c>
-      <c r="M10" s="33" t="n">
-        <v>-0.009599999999999999</v>
-      </c>
-      <c r="N10" s="34" t="n">
-        <v>-0.23</v>
-      </c>
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>3PP配件營業額</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="n"/>
+      <c r="C10" s="29" t="n"/>
+      <c r="D10" s="30" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="29" t="n"/>
+      <c r="G10" s="110" t="n"/>
+      <c r="H10" s="31" t="n"/>
+      <c r="I10" s="29" t="n"/>
+      <c r="J10" s="30" t="n"/>
+      <c r="K10" s="31" t="n"/>
+      <c r="L10" s="29" t="n"/>
+      <c r="M10" s="30" t="n"/>
+      <c r="N10" s="31" t="n"/>
     </row>
     <row r="11" ht="34" customHeight="1" s="106">
-      <c r="A11" s="20" t="inlineStr">
-        <is>
-          <t>總毛利額</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="n">
-        <v>165923</v>
-      </c>
-      <c r="C11" s="29" t="n">
-        <v>254070</v>
-      </c>
-      <c r="D11" s="30" t="n">
-        <v>-29608</v>
-      </c>
-      <c r="E11" s="31" t="n">
-        <v>-0.09</v>
-      </c>
-      <c r="F11" s="29" t="n">
-        <v>419993</v>
-      </c>
-      <c r="G11" s="110" t="n"/>
-      <c r="H11" s="31" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="I11" s="29" t="n"/>
-      <c r="J11" s="30" t="n">
-        <v>-509490</v>
-      </c>
-      <c r="K11" s="31" t="n">
-        <v>-0.27</v>
-      </c>
-      <c r="L11" s="29" t="n">
-        <v>343378</v>
-      </c>
-      <c r="M11" s="30" t="n">
-        <v>349578</v>
-      </c>
-      <c r="N11" s="31" t="n">
-        <v>0.34</v>
-      </c>
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>3PP搭售率</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="n"/>
+      <c r="C11" s="33" t="n"/>
+      <c r="D11" s="33" t="n"/>
+      <c r="E11" s="34" t="n"/>
+      <c r="F11" s="33" t="n"/>
+      <c r="G11" s="33" t="n"/>
+      <c r="H11" s="31" t="n"/>
+      <c r="I11" s="33" t="n"/>
+      <c r="J11" s="33" t="n"/>
+      <c r="K11" s="34" t="n"/>
+      <c r="L11" s="33" t="n"/>
+      <c r="M11" s="33" t="n"/>
+      <c r="N11" s="34" t="n"/>
     </row>
     <row r="12" ht="34" customHeight="1" s="106">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>Apple 毛利額</t>
-        </is>
-      </c>
-      <c r="B12" s="29" t="n">
-        <v>87950</v>
-      </c>
-      <c r="C12" s="29" t="n">
-        <v>113767</v>
-      </c>
-      <c r="D12" s="30" t="n">
-        <v>-10364</v>
-      </c>
-      <c r="E12" s="31" t="n">
-        <v>-0.07000000000000001</v>
-      </c>
-      <c r="F12" s="29" t="n">
-        <v>201717</v>
-      </c>
+          <t>ACPP 營業額</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="n"/>
+      <c r="C12" s="29" t="n"/>
+      <c r="D12" s="30" t="n"/>
+      <c r="E12" s="31" t="n"/>
+      <c r="F12" s="29" t="n"/>
       <c r="G12" s="110" t="n"/>
-      <c r="H12" s="31" t="n">
-        <v>1.02</v>
-      </c>
+      <c r="H12" s="31" t="n"/>
       <c r="I12" s="29" t="n"/>
-      <c r="J12" s="30" t="n">
-        <v>-369579</v>
-      </c>
-      <c r="K12" s="31" t="n">
-        <v>-0.36</v>
-      </c>
-      <c r="L12" s="29" t="n">
-        <v>193985</v>
-      </c>
-      <c r="M12" s="30" t="n">
-        <v>78923</v>
-      </c>
-      <c r="N12" s="31" t="n">
-        <v>0.14</v>
-      </c>
+      <c r="J12" s="30" t="n"/>
+      <c r="K12" s="31" t="n"/>
+      <c r="L12" s="29" t="n"/>
+      <c r="M12" s="30" t="n"/>
+      <c r="N12" s="31" t="n"/>
     </row>
     <row r="13" ht="34" customHeight="1" s="106">
-      <c r="A13" s="20" t="inlineStr">
-        <is>
-          <t>3PP 毛利額</t>
-        </is>
-      </c>
-      <c r="B13" s="29" t="n">
-        <v>53698</v>
-      </c>
-      <c r="C13" s="29" t="n">
-        <v>107243</v>
-      </c>
-      <c r="D13" s="30" t="n">
-        <v>-13544</v>
-      </c>
-      <c r="E13" s="31" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="F13" s="29" t="n">
-        <v>160941</v>
-      </c>
-      <c r="G13" s="110" t="n"/>
-      <c r="H13" s="31" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="I13" s="29" t="n"/>
-      <c r="J13" s="30" t="n">
-        <v>-13681</v>
-      </c>
-      <c r="K13" s="31" t="n">
-        <v>-0.02</v>
-      </c>
-      <c r="L13" s="29" t="n">
-        <v>72668</v>
-      </c>
-      <c r="M13" s="30" t="n">
-        <v>281475</v>
-      </c>
-      <c r="N13" s="31" t="n">
-        <v>0.9399999999999999</v>
-      </c>
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>ACPP 搭售率</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="n"/>
+      <c r="C13" s="33" t="n"/>
+      <c r="D13" s="33" t="n"/>
+      <c r="E13" s="34" t="n"/>
+      <c r="F13" s="33" t="n"/>
+      <c r="G13" s="33" t="n"/>
+      <c r="H13" s="31" t="n"/>
+      <c r="I13" s="33" t="n"/>
+      <c r="J13" s="33" t="n"/>
+      <c r="K13" s="34" t="n"/>
+      <c r="L13" s="33" t="n"/>
+      <c r="M13" s="33" t="n"/>
+      <c r="N13" s="34" t="n"/>
     </row>
     <row r="14" ht="34" customHeight="1" s="106">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>SA Care 毛利額</t>
-        </is>
-      </c>
-      <c r="B14" s="29" t="n">
-        <v>24275</v>
-      </c>
-      <c r="C14" s="29" t="n">
-        <v>33060</v>
-      </c>
-      <c r="D14" s="30" t="n">
-        <v>-5700</v>
-      </c>
-      <c r="E14" s="31" t="n">
-        <v>-0.13</v>
-      </c>
-      <c r="F14" s="29" t="n">
-        <v>57335</v>
-      </c>
+          <t>SA Care 營業額(e)</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="n"/>
+      <c r="C14" s="29" t="n"/>
+      <c r="D14" s="30" t="n"/>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="29" t="n"/>
       <c r="G14" s="110" t="n"/>
-      <c r="H14" s="31" t="n">
-        <v>0.86</v>
-      </c>
+      <c r="H14" s="31" t="n"/>
       <c r="I14" s="29" t="n"/>
-      <c r="J14" s="30" t="n">
-        <v>-126230</v>
-      </c>
-      <c r="K14" s="31" t="n">
-        <v>-0.45</v>
-      </c>
-      <c r="L14" s="29" t="n">
-        <v>76725</v>
-      </c>
-      <c r="M14" s="30" t="n">
-        <v>-10820</v>
-      </c>
-      <c r="N14" s="31" t="n">
-        <v>-0.07000000000000001</v>
-      </c>
+      <c r="J14" s="30" t="n"/>
+      <c r="K14" s="31" t="n"/>
+      <c r="L14" s="29" t="n"/>
+      <c r="M14" s="30" t="n"/>
+      <c r="N14" s="31" t="n"/>
     </row>
     <row r="15" ht="34" customHeight="1" s="106">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>CPU 台數（不含Mac mini）</t>
-        </is>
-      </c>
-      <c r="B15" s="29" t="n"/>
-      <c r="C15" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" s="30" t="n">
-        <v>-1</v>
-      </c>
-      <c r="E15" s="31" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F15" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="G15" s="110" t="n"/>
-      <c r="H15" s="31" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="I15" s="29" t="n"/>
-      <c r="J15" s="30" t="n">
-        <v>-4</v>
-      </c>
-      <c r="K15" s="31" t="n">
-        <v>-0.27</v>
-      </c>
-      <c r="L15" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="M15" s="30" t="n">
-        <v>-2</v>
-      </c>
-      <c r="N15" s="31" t="n">
-        <v>-0.15</v>
-      </c>
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>SA Care 搭售率</t>
+        </is>
+      </c>
+      <c r="B15" s="33" t="n"/>
+      <c r="C15" s="33" t="n"/>
+      <c r="D15" s="33" t="n"/>
+      <c r="E15" s="34" t="n"/>
+      <c r="F15" s="33" t="n"/>
+      <c r="G15" s="33" t="n"/>
+      <c r="H15" s="31" t="n"/>
+      <c r="I15" s="33" t="n"/>
+      <c r="J15" s="33" t="n"/>
+      <c r="K15" s="34" t="n"/>
+      <c r="L15" s="33" t="n"/>
+      <c r="M15" s="33" t="n"/>
+      <c r="N15" s="34" t="n"/>
     </row>
     <row r="16" ht="34" customHeight="1" s="106">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>Mac mini 台數</t>
-        </is>
-      </c>
-      <c r="B16" s="35" t="n"/>
-      <c r="C16" s="35" t="n"/>
-      <c r="D16" s="32" t="n"/>
-      <c r="E16" s="32" t="n"/>
+          <t>總毛利額</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="n"/>
+      <c r="C16" s="29" t="n"/>
+      <c r="D16" s="30" t="n"/>
+      <c r="E16" s="31" t="n"/>
       <c r="F16" s="29" t="n"/>
       <c r="G16" s="110" t="n"/>
-      <c r="H16" s="31" t="n">
-        <v>5</v>
-      </c>
+      <c r="H16" s="31" t="n"/>
       <c r="I16" s="29" t="n"/>
-      <c r="J16" s="30" t="n">
-        <v>8</v>
-      </c>
-      <c r="K16" s="31" t="n">
-        <v>4</v>
-      </c>
-      <c r="L16" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="M16" s="30" t="n">
-        <v>7</v>
-      </c>
-      <c r="N16" s="31" t="n">
-        <v>2.33</v>
-      </c>
+      <c r="J16" s="30" t="n"/>
+      <c r="K16" s="31" t="n"/>
+      <c r="L16" s="29" t="n"/>
+      <c r="M16" s="30" t="n"/>
+      <c r="N16" s="31" t="n"/>
     </row>
     <row r="17" ht="34" customHeight="1" s="106">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>CPU 總台數</t>
+          <t>Apple 毛利額</t>
         </is>
       </c>
       <c r="B17" s="29" t="n"/>
-      <c r="C17" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="30" t="n">
-        <v>-1</v>
-      </c>
-      <c r="E17" s="31" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F17" s="29" t="n">
-        <v>2</v>
-      </c>
+      <c r="C17" s="29" t="n"/>
+      <c r="D17" s="30" t="n"/>
+      <c r="E17" s="31" t="n"/>
+      <c r="F17" s="29" t="n"/>
       <c r="G17" s="110" t="n"/>
-      <c r="H17" s="31" t="n">
-        <v>1.29</v>
-      </c>
+      <c r="H17" s="31" t="n"/>
       <c r="I17" s="29" t="n"/>
-      <c r="J17" s="30" t="n">
-        <v>4</v>
-      </c>
-      <c r="K17" s="31" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="L17" s="29" t="n">
-        <v>5</v>
-      </c>
-      <c r="M17" s="30" t="n">
-        <v>5</v>
-      </c>
-      <c r="N17" s="31" t="n">
-        <v>0.31</v>
-      </c>
+      <c r="J17" s="30" t="n"/>
+      <c r="K17" s="31" t="n"/>
+      <c r="L17" s="29" t="n"/>
+      <c r="M17" s="30" t="n"/>
+      <c r="N17" s="31" t="n"/>
     </row>
     <row r="18" ht="34" customHeight="1" s="106">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>ACPP-MAC 套數</t>
-        </is>
-      </c>
-      <c r="B18" s="35" t="n"/>
-      <c r="C18" s="35" t="n"/>
-      <c r="D18" s="32" t="n"/>
-      <c r="E18" s="32" t="n"/>
+          <t>3PP 毛利額</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="n"/>
+      <c r="C18" s="29" t="n"/>
+      <c r="D18" s="30" t="n"/>
+      <c r="E18" s="31" t="n"/>
       <c r="F18" s="29" t="n"/>
       <c r="G18" s="110" t="n"/>
-      <c r="H18" s="31" t="n">
-        <v>1</v>
-      </c>
+      <c r="H18" s="31" t="n"/>
       <c r="I18" s="29" t="n"/>
-      <c r="J18" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="L18" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="M18" s="30" t="n">
-        <v>-2</v>
-      </c>
-      <c r="N18" s="31" t="n">
-        <v>-0.5</v>
-      </c>
+      <c r="J18" s="30" t="n"/>
+      <c r="K18" s="31" t="n"/>
+      <c r="L18" s="29" t="n"/>
+      <c r="M18" s="30" t="n"/>
+      <c r="N18" s="31" t="n"/>
     </row>
     <row r="19" ht="34" customHeight="1" s="106">
-      <c r="A19" s="27" t="inlineStr">
-        <is>
-          <t>ACPP-MAC 搭售率</t>
-        </is>
-      </c>
-      <c r="B19" s="111" t="n"/>
-      <c r="C19" s="112" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="36" t="n"/>
-      <c r="E19" s="36" t="n"/>
-      <c r="F19" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="34" t="n"/>
-      <c r="H19" s="31" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="I19" s="33" t="n"/>
-      <c r="J19" s="33" t="n">
-        <v>0.1152</v>
-      </c>
-      <c r="K19" s="34" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="L19" s="33" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M19" s="33" t="n">
-        <v>-0.1259</v>
-      </c>
-      <c r="N19" s="34" t="n">
-        <v>-0.41</v>
-      </c>
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>ACPP毛利額</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="n"/>
+      <c r="C19" s="29" t="n"/>
+      <c r="D19" s="30" t="n"/>
+      <c r="E19" s="31" t="n"/>
+      <c r="F19" s="29" t="n"/>
+      <c r="G19" s="110" t="n"/>
+      <c r="H19" s="31" t="n"/>
+      <c r="I19" s="29" t="n"/>
+      <c r="J19" s="30" t="n"/>
+      <c r="K19" s="31" t="n"/>
+      <c r="L19" s="29" t="n"/>
+      <c r="M19" s="30" t="n"/>
+      <c r="N19" s="31" t="n"/>
     </row>
     <row r="20" ht="34" customHeight="1" s="106">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>SA Care for CPU 套數</t>
+          <t>SA Care 毛利額</t>
         </is>
       </c>
       <c r="B20" s="29" t="n"/>
-      <c r="C20" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="30" t="n">
-        <v>-1</v>
-      </c>
-      <c r="E20" s="31" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F20" s="29" t="n">
-        <v>1</v>
-      </c>
+      <c r="C20" s="29" t="n"/>
+      <c r="D20" s="30" t="n"/>
+      <c r="E20" s="31" t="n"/>
+      <c r="F20" s="29" t="n"/>
       <c r="G20" s="110" t="n"/>
-      <c r="H20" s="31" t="n">
-        <v>0.5600000000000001</v>
-      </c>
+      <c r="H20" s="31" t="n"/>
       <c r="I20" s="29" t="n"/>
-      <c r="J20" s="32" t="n"/>
-      <c r="K20" s="32" t="n"/>
-      <c r="L20" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="M20" s="30" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N20" s="31" t="n">
-        <v>-0.17</v>
-      </c>
+      <c r="J20" s="30" t="n"/>
+      <c r="K20" s="31" t="n"/>
+      <c r="L20" s="29" t="n"/>
+      <c r="M20" s="30" t="n"/>
+      <c r="N20" s="31" t="n"/>
     </row>
     <row r="21" ht="34" customHeight="1" s="106">
-      <c r="A21" s="27" t="inlineStr">
-        <is>
-          <t>SA Care for CPU 搭售率</t>
-        </is>
-      </c>
-      <c r="B21" s="111" t="n"/>
-      <c r="C21" s="112" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D21" s="36" t="n"/>
-      <c r="E21" s="36" t="n"/>
-      <c r="F21" s="33" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G21" s="34" t="n"/>
-      <c r="H21" s="31" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="I21" s="33" t="n"/>
-      <c r="J21" s="33" t="n">
-        <v>-0.056</v>
-      </c>
-      <c r="K21" s="34" t="n">
-        <v>-0.19</v>
-      </c>
-      <c r="L21" s="33" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M21" s="33" t="n">
-        <v>-0.1369</v>
-      </c>
-      <c r="N21" s="34" t="n">
-        <v>-0.37</v>
-      </c>
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>CPU 台數</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="n"/>
+      <c r="C21" s="35" t="n"/>
+      <c r="D21" s="30" t="n"/>
+      <c r="E21" s="31" t="n"/>
+      <c r="F21" s="29" t="n"/>
+      <c r="G21" s="110" t="n"/>
+      <c r="H21" s="31" t="n"/>
+      <c r="I21" s="29" t="n"/>
+      <c r="J21" s="30" t="n"/>
+      <c r="K21" s="31" t="n"/>
+      <c r="L21" s="29" t="n"/>
+      <c r="M21" s="30" t="n"/>
+      <c r="N21" s="31" t="n"/>
     </row>
     <row r="22" ht="34" customHeight="1" s="106">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>iPad 台數</t>
-        </is>
-      </c>
-      <c r="B22" s="29" t="n">
-        <v>13</v>
-      </c>
-      <c r="C22" s="29" t="n">
-        <v>10</v>
-      </c>
-      <c r="D22" s="30" t="n">
-        <v>8</v>
-      </c>
-      <c r="E22" s="31" t="n">
-        <v>0.89</v>
-      </c>
-      <c r="F22" s="29" t="n">
-        <v>23</v>
-      </c>
+          <t>ACPP-MAC 套數</t>
+        </is>
+      </c>
+      <c r="B22" s="35" t="n"/>
+      <c r="C22" s="35" t="n"/>
+      <c r="D22" s="32" t="n"/>
+      <c r="E22" s="32" t="n"/>
+      <c r="F22" s="29" t="n"/>
       <c r="G22" s="110" t="n"/>
-      <c r="H22" s="31" t="n">
-        <v>1.05</v>
-      </c>
+      <c r="H22" s="31" t="n"/>
       <c r="I22" s="29" t="n"/>
-      <c r="J22" s="30" t="n">
-        <v>-35</v>
-      </c>
-      <c r="K22" s="31" t="n">
-        <v>-0.44</v>
-      </c>
-      <c r="L22" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="M22" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="N22" s="31" t="n">
-        <v>0.05</v>
-      </c>
+      <c r="J22" s="30" t="n"/>
+      <c r="K22" s="31" t="n"/>
+      <c r="L22" s="29" t="n"/>
+      <c r="M22" s="30" t="n"/>
+      <c r="N22" s="31" t="n"/>
     </row>
     <row r="23" ht="34" customHeight="1" s="106">
       <c r="A23" s="20" t="inlineStr">
         <is>
-          <t>SA Care for iPad 套數</t>
-        </is>
-      </c>
-      <c r="B23" s="29" t="n">
-        <v>8</v>
-      </c>
-      <c r="C23" s="29" t="n">
-        <v>9</v>
-      </c>
-      <c r="D23" s="30" t="n">
-        <v>6</v>
-      </c>
-      <c r="E23" s="31" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" s="29" t="n">
-        <v>17</v>
-      </c>
+          <t>SA Care for CPU 套數</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="n"/>
+      <c r="C23" s="35" t="n"/>
+      <c r="D23" s="30" t="n"/>
+      <c r="E23" s="31" t="n"/>
+      <c r="F23" s="29" t="n"/>
       <c r="G23" s="110" t="n"/>
-      <c r="H23" s="31" t="n">
-        <v>0.86</v>
-      </c>
+      <c r="H23" s="31" t="n"/>
       <c r="I23" s="29" t="n"/>
-      <c r="J23" s="30" t="n">
-        <v>-20</v>
-      </c>
-      <c r="K23" s="31" t="n">
-        <v>-0.51</v>
-      </c>
-      <c r="L23" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="M23" s="30" t="n">
-        <v>-5</v>
-      </c>
-      <c r="N23" s="31" t="n">
-        <v>-0.21</v>
-      </c>
+      <c r="J23" s="32" t="n"/>
+      <c r="K23" s="32" t="n"/>
+      <c r="L23" s="29" t="n"/>
+      <c r="M23" s="30" t="n"/>
+      <c r="N23" s="31" t="n"/>
     </row>
     <row r="24" ht="34" customHeight="1" s="106">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>SA Care for iPad 搭售率</t>
-        </is>
-      </c>
-      <c r="B24" s="111" t="n">
-        <v>0.6153999999999999</v>
-      </c>
-      <c r="C24" s="111" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="D24" s="111" t="n">
-        <v>0.1961</v>
-      </c>
-      <c r="E24" s="34" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="F24" s="33" t="n">
-        <v>0.7391</v>
-      </c>
+          <t>保固加總 CPU 搭售率</t>
+        </is>
+      </c>
+      <c r="B24" s="34" t="n"/>
+      <c r="C24" s="185" t="n"/>
+      <c r="D24" s="185" t="n"/>
+      <c r="E24" s="36" t="n"/>
+      <c r="F24" s="34" t="n"/>
       <c r="G24" s="34" t="n"/>
-      <c r="H24" s="31" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="I24" s="33" t="n"/>
-      <c r="J24" s="33" t="n">
-        <v>-0.0653</v>
-      </c>
-      <c r="K24" s="34" t="n">
-        <v>-0.13</v>
-      </c>
-      <c r="L24" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="M24" s="33" t="n">
-        <v>-0.1359</v>
-      </c>
-      <c r="N24" s="34" t="n">
-        <v>-0.24</v>
-      </c>
+      <c r="H24" s="31" t="n"/>
+      <c r="I24" s="34" t="n"/>
+      <c r="J24" s="34" t="n"/>
+      <c r="K24" s="34" t="n"/>
+      <c r="L24" s="34" t="n"/>
+      <c r="M24" s="34" t="n"/>
+      <c r="N24" s="34" t="n"/>
     </row>
     <row r="25" ht="34" customHeight="1" s="106">
       <c r="A25" s="20" t="inlineStr">
         <is>
-          <t>iPhone 台數</t>
-        </is>
-      </c>
-      <c r="B25" s="29" t="n">
-        <v>18</v>
-      </c>
-      <c r="C25" s="29" t="n">
-        <v>21</v>
-      </c>
-      <c r="D25" s="30" t="n">
-        <v>-15</v>
-      </c>
-      <c r="E25" s="31" t="n">
-        <v>-0.32</v>
-      </c>
-      <c r="F25" s="29" t="n">
-        <v>39</v>
-      </c>
+          <t>iPad 台數</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="n"/>
+      <c r="C25" s="29" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31" t="n"/>
+      <c r="F25" s="29" t="n"/>
       <c r="G25" s="110" t="n"/>
-      <c r="H25" s="31" t="n">
-        <v>1.44</v>
-      </c>
+      <c r="H25" s="31" t="n"/>
       <c r="I25" s="29" t="n"/>
-      <c r="J25" s="30" t="n">
-        <v>-53</v>
-      </c>
-      <c r="K25" s="31" t="n">
-        <v>-0.26</v>
-      </c>
+      <c r="J25" s="30" t="n"/>
+      <c r="K25" s="31" t="n"/>
       <c r="L25" s="29" t="n"/>
-      <c r="M25" s="30" t="n">
-        <v>50</v>
-      </c>
-      <c r="N25" s="31" t="n">
-        <v>0.51</v>
-      </c>
+      <c r="M25" s="30" t="n"/>
+      <c r="N25" s="31" t="n"/>
     </row>
     <row r="26" ht="34" customHeight="1" s="106">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>SA Care for iPhone 套數</t>
-        </is>
-      </c>
-      <c r="B26" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="C26" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="D26" s="30" t="n">
-        <v>-4</v>
-      </c>
-      <c r="E26" s="31" t="n">
-        <v>-0.33</v>
-      </c>
-      <c r="F26" s="29" t="n">
-        <v>8</v>
-      </c>
+          <t>ACPP-iPad 套數</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="n"/>
+      <c r="C26" s="29" t="n"/>
+      <c r="D26" s="30" t="n"/>
+      <c r="E26" s="31" t="n"/>
+      <c r="F26" s="29" t="n"/>
       <c r="G26" s="110" t="n"/>
-      <c r="H26" s="31" t="n">
-        <v>1.55</v>
-      </c>
+      <c r="H26" s="31" t="n"/>
       <c r="I26" s="29" t="n"/>
-      <c r="J26" s="30" t="n">
-        <v>-25</v>
-      </c>
-      <c r="K26" s="31" t="n">
-        <v>-0.45</v>
-      </c>
-      <c r="L26" s="29" t="n">
-        <v>20</v>
-      </c>
-      <c r="M26" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="N26" s="31" t="n">
-        <v>0.11</v>
-      </c>
+      <c r="J26" s="30" t="n"/>
+      <c r="K26" s="31" t="n"/>
+      <c r="L26" s="29" t="n"/>
+      <c r="M26" s="30" t="n"/>
+      <c r="N26" s="31" t="n"/>
     </row>
     <row r="27" ht="34" customHeight="1" s="106">
-      <c r="A27" s="27" t="inlineStr">
-        <is>
-          <t>SA Care for iPhone 搭售率</t>
-        </is>
-      </c>
-      <c r="B27" s="33" t="n">
-        <v>0.2222</v>
-      </c>
-      <c r="C27" s="33" t="n">
-        <v>0.1905</v>
-      </c>
-      <c r="D27" s="33" t="n">
-        <v>-0.0053</v>
-      </c>
-      <c r="E27" s="34" t="n">
-        <v>-0.02</v>
-      </c>
-      <c r="F27" s="33" t="n">
-        <v>0.2051</v>
-      </c>
-      <c r="G27" s="34" t="n"/>
-      <c r="H27" s="31" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="I27" s="33" t="n"/>
-      <c r="J27" s="33" t="n">
-        <v>-0.0692</v>
-      </c>
-      <c r="K27" s="34" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="L27" s="33" t="n"/>
-      <c r="M27" s="33" t="n">
-        <v>-0.07480000000000001</v>
-      </c>
-      <c r="N27" s="34" t="n">
-        <v>-0.26</v>
-      </c>
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>SA Care for iPad 套數</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="n"/>
+      <c r="C27" s="29" t="n"/>
+      <c r="D27" s="30" t="n"/>
+      <c r="E27" s="31" t="n"/>
+      <c r="F27" s="29" t="n"/>
+      <c r="G27" s="110" t="n"/>
+      <c r="H27" s="31" t="n"/>
+      <c r="I27" s="29" t="n"/>
+      <c r="J27" s="30" t="n"/>
+      <c r="K27" s="31" t="n"/>
+      <c r="L27" s="29" t="n"/>
+      <c r="M27" s="30" t="n"/>
+      <c r="N27" s="31" t="n"/>
     </row>
     <row r="28" ht="34" customHeight="1" s="106">
-      <c r="A28" s="20" t="inlineStr">
-        <is>
-          <t>Watch 台數</t>
-        </is>
-      </c>
-      <c r="B28" s="29" t="n">
-        <v>5</v>
-      </c>
-      <c r="C28" s="29" t="n">
-        <v>8</v>
-      </c>
-      <c r="D28" s="30" t="n">
-        <v>4</v>
-      </c>
-      <c r="E28" s="31" t="n">
-        <v>2</v>
-      </c>
-      <c r="F28" s="29" t="n">
-        <v>13</v>
-      </c>
-      <c r="G28" s="110" t="n"/>
-      <c r="H28" s="31" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="I28" s="29" t="n"/>
-      <c r="J28" s="30" t="n">
-        <v>-43</v>
-      </c>
-      <c r="K28" s="31" t="n">
-        <v>-0.54</v>
-      </c>
-      <c r="L28" s="29" t="n"/>
-      <c r="M28" s="30" t="n">
-        <v>-17</v>
-      </c>
-      <c r="N28" s="31" t="n">
-        <v>-0.31</v>
-      </c>
+      <c r="A28" s="27" t="inlineStr">
+        <is>
+          <t>保固加總 iPad 搭售率</t>
+        </is>
+      </c>
+      <c r="B28" s="34" t="n"/>
+      <c r="C28" s="34" t="n"/>
+      <c r="D28" s="34" t="n"/>
+      <c r="E28" s="34" t="n"/>
+      <c r="F28" s="34" t="n"/>
+      <c r="G28" s="34" t="n"/>
+      <c r="H28" s="31" t="n"/>
+      <c r="I28" s="34" t="n"/>
+      <c r="J28" s="34" t="n"/>
+      <c r="K28" s="34" t="n"/>
+      <c r="L28" s="34" t="n"/>
+      <c r="M28" s="34" t="n"/>
+      <c r="N28" s="34" t="n"/>
     </row>
     <row r="29" ht="34" customHeight="1" s="106">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>SA Care for Watch 套數</t>
-        </is>
-      </c>
-      <c r="B29" s="35" t="n">
-        <v>3</v>
-      </c>
-      <c r="C29" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="D29" s="30" t="n">
-        <v>4</v>
-      </c>
-      <c r="E29" s="32" t="n"/>
-      <c r="F29" s="29" t="n">
-        <v>6</v>
-      </c>
+          <t>iPhone 台數</t>
+        </is>
+      </c>
+      <c r="B29" s="29" t="n"/>
+      <c r="C29" s="29" t="n"/>
+      <c r="D29" s="30" t="n"/>
+      <c r="E29" s="31" t="n"/>
+      <c r="F29" s="29" t="n"/>
       <c r="G29" s="110" t="n"/>
-      <c r="H29" s="31" t="n">
-        <v>0.64</v>
-      </c>
+      <c r="H29" s="31" t="n"/>
       <c r="I29" s="29" t="n"/>
-      <c r="J29" s="30" t="n">
-        <v>-24</v>
-      </c>
-      <c r="K29" s="31" t="n">
-        <v>-0.63</v>
-      </c>
-      <c r="L29" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="M29" s="30" t="n">
-        <v>-3</v>
-      </c>
-      <c r="N29" s="31" t="n">
-        <v>-0.18</v>
-      </c>
+      <c r="J29" s="30" t="n"/>
+      <c r="K29" s="31" t="n"/>
+      <c r="L29" s="29" t="n"/>
+      <c r="M29" s="30" t="n"/>
+      <c r="N29" s="31" t="n"/>
     </row>
     <row r="30" ht="34" customHeight="1" s="106">
-      <c r="A30" s="27" t="inlineStr">
-        <is>
-          <t>SA Care for Watch 搭售率</t>
-        </is>
-      </c>
-      <c r="B30" s="33" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C30" s="33" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="D30" s="33" t="n">
-        <v>0.6667</v>
-      </c>
-      <c r="E30" s="36" t="n"/>
-      <c r="F30" s="33" t="n">
-        <v>0.4615</v>
-      </c>
-      <c r="G30" s="34" t="n"/>
-      <c r="H30" s="31" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="I30" s="33" t="n"/>
-      <c r="J30" s="33" t="n">
-        <v>-0.09660000000000001</v>
-      </c>
-      <c r="K30" s="34" t="n">
-        <v>-0.2</v>
-      </c>
-      <c r="L30" s="33" t="n"/>
-      <c r="M30" s="33" t="n">
-        <v>0.0636</v>
-      </c>
-      <c r="N30" s="34" t="n">
-        <v>0.2</v>
-      </c>
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>ACPP-iPhone 套數</t>
+        </is>
+      </c>
+      <c r="B30" s="29" t="n"/>
+      <c r="C30" s="29" t="n"/>
+      <c r="D30" s="30" t="n"/>
+      <c r="E30" s="31" t="n"/>
+      <c r="F30" s="29" t="n"/>
+      <c r="G30" s="110" t="n"/>
+      <c r="H30" s="31" t="n"/>
+      <c r="I30" s="29" t="n"/>
+      <c r="J30" s="30" t="n"/>
+      <c r="K30" s="31" t="n"/>
+      <c r="L30" s="29" t="n"/>
+      <c r="M30" s="30" t="n"/>
+      <c r="N30" s="31" t="n"/>
     </row>
     <row r="31" ht="34" customHeight="1" s="106">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>人均產值</t>
-        </is>
-      </c>
-      <c r="B31" s="100" t="n"/>
-      <c r="C31" s="100" t="n"/>
-      <c r="D31" s="101" t="n">
-        <v>100000</v>
-      </c>
-      <c r="E31" s="31" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="F31" s="100" t="n"/>
-      <c r="G31" s="32" t="n"/>
-      <c r="H31" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="100" t="n"/>
-      <c r="J31" s="101" t="n">
-        <v>-800000</v>
-      </c>
-      <c r="K31" s="31" t="n">
-        <v>-0.32</v>
-      </c>
-      <c r="L31" s="100" t="n"/>
-      <c r="M31" s="101" t="n">
-        <v>300000</v>
-      </c>
-      <c r="N31" s="31" t="n">
-        <v>0.23</v>
-      </c>
+          <t>SA Care for iPhone 套數</t>
+        </is>
+      </c>
+      <c r="B31" s="29" t="n"/>
+      <c r="C31" s="29" t="n"/>
+      <c r="D31" s="30" t="n"/>
+      <c r="E31" s="31" t="n"/>
+      <c r="F31" s="29" t="n"/>
+      <c r="G31" s="110" t="n"/>
+      <c r="H31" s="31" t="n"/>
+      <c r="I31" s="29" t="n"/>
+      <c r="J31" s="30" t="n"/>
+      <c r="K31" s="31" t="n"/>
+      <c r="L31" s="29" t="n"/>
+      <c r="M31" s="30" t="n"/>
+      <c r="N31" s="31" t="n"/>
     </row>
     <row r="32" ht="34" customHeight="1" s="106">
-      <c r="A32" s="20" t="inlineStr">
-        <is>
-          <t>來客數</t>
-        </is>
-      </c>
-      <c r="B32" s="100" t="n"/>
-      <c r="C32" s="100" t="n"/>
-      <c r="D32" s="101" t="n">
-        <v>-200</v>
-      </c>
-      <c r="E32" s="31" t="n">
-        <v>-0.14</v>
-      </c>
-      <c r="F32" s="100" t="n"/>
-      <c r="G32" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="29" t="n"/>
-      <c r="J32" s="101" t="n">
-        <v>-500</v>
-      </c>
-      <c r="K32" s="31" t="n">
-        <v>-0.08</v>
-      </c>
-      <c r="L32" s="100" t="n"/>
-      <c r="M32" s="101" t="n">
-        <v>-900</v>
-      </c>
-      <c r="N32" s="31" t="n">
-        <v>-0.13</v>
-      </c>
+      <c r="A32" s="27" t="inlineStr">
+        <is>
+          <t>保固加總 iPhone 搭售率</t>
+        </is>
+      </c>
+      <c r="B32" s="34" t="n"/>
+      <c r="C32" s="34" t="n"/>
+      <c r="D32" s="34" t="n"/>
+      <c r="E32" s="34" t="n"/>
+      <c r="F32" s="34" t="n"/>
+      <c r="G32" s="34" t="n"/>
+      <c r="H32" s="31" t="n"/>
+      <c r="I32" s="34" t="n"/>
+      <c r="J32" s="34" t="n"/>
+      <c r="K32" s="34" t="n"/>
+      <c r="L32" s="34" t="n"/>
+      <c r="M32" s="34" t="n"/>
+      <c r="N32" s="34" t="n"/>
     </row>
     <row r="33" ht="34" customHeight="1" s="106">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>成交筆數</t>
+          <t>Watch 台數</t>
         </is>
       </c>
       <c r="B33" s="29" t="n"/>
@@ -9868,64 +9264,234 @@
       <c r="D33" s="30" t="n"/>
       <c r="E33" s="31" t="n"/>
       <c r="F33" s="29" t="n"/>
-      <c r="G33" s="30" t="n"/>
+      <c r="G33" s="110" t="n"/>
       <c r="H33" s="31" t="n"/>
       <c r="I33" s="29" t="n"/>
       <c r="J33" s="30" t="n"/>
       <c r="K33" s="31" t="n"/>
       <c r="L33" s="29" t="n"/>
-      <c r="M33" s="30" t="n">
-        <v>81</v>
-      </c>
-      <c r="N33" s="31" t="n">
-        <v>0.08</v>
-      </c>
+      <c r="M33" s="30" t="n"/>
+      <c r="N33" s="31" t="n"/>
     </row>
     <row r="34" ht="34" customHeight="1" s="106">
-      <c r="A34" s="28" t="inlineStr">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>ACPP-Watch 套數</t>
+        </is>
+      </c>
+      <c r="B34" s="35" t="n"/>
+      <c r="C34" s="29" t="n"/>
+      <c r="D34" s="30" t="n"/>
+      <c r="E34" s="32" t="n"/>
+      <c r="F34" s="29" t="n"/>
+      <c r="G34" s="110" t="n"/>
+      <c r="H34" s="31" t="n"/>
+      <c r="I34" s="29" t="n"/>
+      <c r="J34" s="30" t="n"/>
+      <c r="K34" s="31" t="n"/>
+      <c r="L34" s="29" t="n"/>
+      <c r="M34" s="30" t="n"/>
+      <c r="N34" s="31" t="n"/>
+    </row>
+    <row r="35" ht="34" customHeight="1" s="106">
+      <c r="A35" s="20" t="inlineStr">
+        <is>
+          <t>SA Care for Watch 套數</t>
+        </is>
+      </c>
+      <c r="B35" s="35" t="n"/>
+      <c r="C35" s="29" t="n"/>
+      <c r="D35" s="30" t="n"/>
+      <c r="E35" s="32" t="n"/>
+      <c r="F35" s="29" t="n"/>
+      <c r="G35" s="110" t="n"/>
+      <c r="H35" s="31" t="n"/>
+      <c r="I35" s="29" t="n"/>
+      <c r="J35" s="30" t="n"/>
+      <c r="K35" s="31" t="n"/>
+      <c r="L35" s="29" t="n"/>
+      <c r="M35" s="30" t="n"/>
+      <c r="N35" s="31" t="n"/>
+    </row>
+    <row r="36" ht="34" customHeight="1" s="106">
+      <c r="A36" s="27" t="inlineStr">
+        <is>
+          <t>保固加總 Watch 搭售率</t>
+        </is>
+      </c>
+      <c r="B36" s="34" t="n"/>
+      <c r="C36" s="34" t="n"/>
+      <c r="D36" s="34" t="n"/>
+      <c r="E36" s="36" t="n"/>
+      <c r="F36" s="34" t="n"/>
+      <c r="G36" s="34" t="n"/>
+      <c r="H36" s="31" t="n"/>
+      <c r="I36" s="34" t="n"/>
+      <c r="J36" s="34" t="n"/>
+      <c r="K36" s="34" t="n"/>
+      <c r="L36" s="34" t="n"/>
+      <c r="M36" s="34" t="n"/>
+      <c r="N36" s="34" t="n"/>
+    </row>
+    <row r="37" ht="34" customHeight="1" s="106">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t>AirPods 台數</t>
+        </is>
+      </c>
+      <c r="B37" s="29" t="n"/>
+      <c r="C37" s="29" t="n"/>
+      <c r="D37" s="30" t="n"/>
+      <c r="E37" s="31" t="n"/>
+      <c r="F37" s="29" t="n"/>
+      <c r="G37" s="110" t="n"/>
+      <c r="H37" s="31" t="n"/>
+      <c r="I37" s="29" t="n"/>
+      <c r="J37" s="30" t="n"/>
+      <c r="K37" s="31" t="n"/>
+      <c r="L37" s="29" t="n"/>
+      <c r="M37" s="30" t="n"/>
+      <c r="N37" s="31" t="n"/>
+    </row>
+    <row r="38" ht="34" customHeight="1" s="106">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>ACPP-AirPods 套數</t>
+        </is>
+      </c>
+      <c r="B38" s="35" t="n"/>
+      <c r="C38" s="29" t="n"/>
+      <c r="D38" s="30" t="n"/>
+      <c r="E38" s="32" t="n"/>
+      <c r="F38" s="29" t="n"/>
+      <c r="G38" s="110" t="n"/>
+      <c r="H38" s="31" t="n"/>
+      <c r="I38" s="29" t="n"/>
+      <c r="J38" s="30" t="n"/>
+      <c r="K38" s="31" t="n"/>
+      <c r="L38" s="29" t="n"/>
+      <c r="M38" s="30" t="n"/>
+      <c r="N38" s="31" t="n"/>
+    </row>
+    <row r="39" ht="34" customHeight="1" s="106">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
+          <t>SA Care for AirPods 套數</t>
+        </is>
+      </c>
+      <c r="B39" s="35" t="n"/>
+      <c r="C39" s="29" t="n"/>
+      <c r="D39" s="30" t="n"/>
+      <c r="E39" s="32" t="n"/>
+      <c r="F39" s="29" t="n"/>
+      <c r="G39" s="110" t="n"/>
+      <c r="H39" s="31" t="n"/>
+      <c r="I39" s="29" t="n"/>
+      <c r="J39" s="30" t="n"/>
+      <c r="K39" s="31" t="n"/>
+      <c r="L39" s="29" t="n"/>
+      <c r="M39" s="30" t="n"/>
+      <c r="N39" s="31" t="n"/>
+    </row>
+    <row r="40" ht="34" customHeight="1" s="106">
+      <c r="A40" s="27" t="inlineStr">
+        <is>
+          <t>保固加總 AirPods 搭售率</t>
+        </is>
+      </c>
+      <c r="B40" s="34" t="n"/>
+      <c r="C40" s="34" t="n"/>
+      <c r="D40" s="34" t="n"/>
+      <c r="E40" s="36" t="n"/>
+      <c r="F40" s="34" t="n"/>
+      <c r="G40" s="34" t="n"/>
+      <c r="H40" s="31" t="n"/>
+      <c r="I40" s="34" t="n"/>
+      <c r="J40" s="34" t="n"/>
+      <c r="K40" s="34" t="n"/>
+      <c r="L40" s="34" t="n"/>
+      <c r="M40" s="34" t="n"/>
+      <c r="N40" s="34" t="n"/>
+    </row>
+    <row r="41" ht="34" customHeight="1" s="106">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>人均產值</t>
+        </is>
+      </c>
+      <c r="B41" s="100" t="n"/>
+      <c r="C41" s="100" t="n"/>
+      <c r="D41" s="101" t="n"/>
+      <c r="E41" s="31" t="n"/>
+      <c r="F41" s="100" t="n"/>
+      <c r="G41" s="32" t="n"/>
+      <c r="H41" s="31" t="n"/>
+      <c r="I41" s="100" t="n"/>
+      <c r="J41" s="101" t="n"/>
+      <c r="K41" s="31" t="n"/>
+      <c r="L41" s="100" t="n"/>
+      <c r="M41" s="101" t="n"/>
+      <c r="N41" s="31" t="n"/>
+    </row>
+    <row r="42" ht="34" customHeight="1" s="106">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>來客數</t>
+        </is>
+      </c>
+      <c r="B42" s="100" t="n"/>
+      <c r="C42" s="100" t="n"/>
+      <c r="D42" s="101" t="n"/>
+      <c r="E42" s="31" t="n"/>
+      <c r="F42" s="100" t="n"/>
+      <c r="G42" s="30" t="n"/>
+      <c r="H42" s="31" t="n"/>
+      <c r="I42" s="29" t="n"/>
+      <c r="J42" s="101" t="n"/>
+      <c r="K42" s="31" t="n"/>
+      <c r="L42" s="100" t="n"/>
+      <c r="M42" s="101" t="n"/>
+      <c r="N42" s="31" t="n"/>
+    </row>
+    <row r="43" ht="34" customHeight="1" s="106">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>成交筆數</t>
+        </is>
+      </c>
+      <c r="B43" s="29" t="n"/>
+      <c r="C43" s="29" t="n"/>
+      <c r="D43" s="30" t="n"/>
+      <c r="E43" s="31" t="n"/>
+      <c r="F43" s="29" t="n"/>
+      <c r="G43" s="30" t="n"/>
+      <c r="H43" s="31" t="n"/>
+      <c r="I43" s="29" t="n"/>
+      <c r="J43" s="30" t="n"/>
+      <c r="K43" s="31" t="n"/>
+      <c r="L43" s="29" t="n"/>
+      <c r="M43" s="30" t="n"/>
+      <c r="N43" s="31" t="n"/>
+    </row>
+    <row r="44" ht="34" customHeight="1" s="106">
+      <c r="A44" s="28" t="inlineStr">
         <is>
           <t>提袋率</t>
         </is>
       </c>
-      <c r="B34" s="37" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="C34" s="37" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="D34" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" s="37" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G34" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" s="37" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="J34" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" s="37" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="M34" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N34" s="31" t="n">
-        <v>0</v>
-      </c>
+      <c r="B44" s="37" t="n"/>
+      <c r="C44" s="37" t="n"/>
+      <c r="D44" s="30" t="n"/>
+      <c r="E44" s="31" t="n"/>
+      <c r="F44" s="37" t="n"/>
+      <c r="G44" s="30" t="n"/>
+      <c r="H44" s="31" t="n"/>
+      <c r="I44" s="37" t="n"/>
+      <c r="J44" s="30" t="n"/>
+      <c r="K44" s="31" t="n"/>
+      <c r="L44" s="37" t="n"/>
+      <c r="M44" s="30" t="n"/>
+      <c r="N44" s="31" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>